<commit_message>
Targets replace the budget: no cap, and reach can earn a richer total
Nothing in the sheet caps a total any more. The single BUDGET cell is
gone, replaced by a per-row TARGET driven by reach: set Y2 for reach 1
and Y3 for reach 2 and every row follows, or overwrite one row for a
one-off. Both ship blank, so CHECK stays quiet until a target is chosen.

Totals no longer need to match across heroes -- splitting the target by
reach is what lets a shorter-reach hero carry better stats.

The 1-50 base range is now a dismissible warning rather than a hard
block, so it guides without getting in the way of tweaking.

Adds a SPREAD read-out at X6:Z10 -- hero count and average total per
reach group -- so the reach/budget trade stays visible while tuning.

Re-verified: 27 heroes, 0 mismatches against MATCHUPS.md, no stat cell
pre-filled.
</commit_message>
<xml_diff>
--- a/resources/characters/hero-stats.xlsx
+++ b/resources/characters/hero-stats.xlsx
@@ -82,11 +82,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -457,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V28"/>
+  <dimension ref="A1:Z28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -482,6 +483,9 @@
     <col width="9" customWidth="1" min="20" max="20"/>
     <col width="15" customWidth="1" min="21" max="21"/>
     <col width="11" customWidth="1" min="22" max="22"/>
+    <col width="30" customWidth="1" min="24" max="24"/>
+    <col width="11" customWidth="1" min="25" max="25"/>
+    <col width="12" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -592,7 +596,12 @@
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>BUDGET</t>
+          <t>TARGET</t>
+        </is>
+      </c>
+      <c r="X1" s="2" t="inlineStr">
+        <is>
+          <t>TARGET TOTAL BY REACH</t>
         </is>
       </c>
     </row>
@@ -625,12 +634,12 @@
           <t>Fire</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Air</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Water</t>
         </is>
@@ -638,27 +647,34 @@
       <c r="I2" t="n">
         <v>1</v>
       </c>
-      <c r="J2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
-      <c r="N2" s="3" t="n"/>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="3" t="n"/>
-      <c r="Q2" s="3" t="n"/>
-      <c r="R2" s="3" t="n"/>
-      <c r="S2" s="3" t="n"/>
-      <c r="T2" s="4">
+      <c r="J2" s="4" t="n"/>
+      <c r="K2" s="4" t="n"/>
+      <c r="L2" s="4" t="n"/>
+      <c r="M2" s="4" t="n"/>
+      <c r="N2" s="4" t="n"/>
+      <c r="O2" s="4" t="n"/>
+      <c r="P2" s="4" t="n"/>
+      <c r="Q2" s="4" t="n"/>
+      <c r="R2" s="4" t="n"/>
+      <c r="S2" s="4" t="n"/>
+      <c r="T2" s="5">
         <f>SUM(J2:S2)</f>
         <v/>
       </c>
       <c r="U2">
-        <f>IF(COUNT(J2:S2)=0,"",IF(COUNT(J2:S2)&lt;10,"INCOMPLETE",IF(T2=$V$2,"OK","OFF BY "&amp;TEXT(T2-$V$2,"+0;-0"))))</f>
-        <v/>
-      </c>
-      <c r="V2" s="4" t="n">
-        <v>250</v>
-      </c>
+        <f>IF(COUNT(J2:S2)=0,"",IF(COUNT(J2:S2)&lt;10,"INCOMPLETE",IF(N(V2)=0,"",IF(T2=V2,"OK","OFF BY "&amp;TEXT(T2-V2,"+0;-0")))))</f>
+        <v/>
+      </c>
+      <c r="V2">
+        <f>IF(N($Y$2)+N($Y$3)=0,"",IF($I2=1,$Y$2,$Y$3))</f>
+        <v/>
+      </c>
+      <c r="X2" s="5" t="inlineStr">
+        <is>
+          <t>Reach 1</t>
+        </is>
+      </c>
+      <c r="Y2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -689,12 +705,12 @@
           <t>Dark</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Air</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Light</t>
         </is>
@@ -702,29 +718,34 @@
       <c r="I3" t="n">
         <v>2</v>
       </c>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="n"/>
-      <c r="M3" s="3" t="n"/>
-      <c r="N3" s="3" t="n"/>
-      <c r="O3" s="3" t="n"/>
-      <c r="P3" s="3" t="n"/>
-      <c r="Q3" s="3" t="n"/>
-      <c r="R3" s="3" t="n"/>
-      <c r="S3" s="3" t="n"/>
-      <c r="T3" s="4">
+      <c r="J3" s="4" t="n"/>
+      <c r="K3" s="4" t="n"/>
+      <c r="L3" s="4" t="n"/>
+      <c r="M3" s="4" t="n"/>
+      <c r="N3" s="4" t="n"/>
+      <c r="O3" s="4" t="n"/>
+      <c r="P3" s="4" t="n"/>
+      <c r="Q3" s="4" t="n"/>
+      <c r="R3" s="4" t="n"/>
+      <c r="S3" s="4" t="n"/>
+      <c r="T3" s="5">
         <f>SUM(J3:S3)</f>
         <v/>
       </c>
       <c r="U3">
-        <f>IF(COUNT(J3:S3)=0,"",IF(COUNT(J3:S3)&lt;10,"INCOMPLETE",IF(T3=$V$2,"OK","OFF BY "&amp;TEXT(T3-$V$2,"+0;-0"))))</f>
-        <v/>
-      </c>
-      <c r="V3" s="5" t="inlineStr">
-        <is>
-          <t>edit V2 only</t>
-        </is>
-      </c>
+        <f>IF(COUNT(J3:S3)=0,"",IF(COUNT(J3:S3)&lt;10,"INCOMPLETE",IF(N(V3)=0,"",IF(T3=V3,"OK","OFF BY "&amp;TEXT(T3-V3,"+0;-0")))))</f>
+        <v/>
+      </c>
+      <c r="V3">
+        <f>IF(N($Y$2)+N($Y$3)=0,"",IF($I3=1,$Y$2,$Y$3))</f>
+        <v/>
+      </c>
+      <c r="X3" s="5" t="inlineStr">
+        <is>
+          <t>Reach 2</t>
+        </is>
+      </c>
+      <c r="Y3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -755,12 +776,12 @@
           <t>Light</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Air</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Dark</t>
         </is>
@@ -768,23 +789,32 @@
       <c r="I4" t="n">
         <v>2</v>
       </c>
-      <c r="J4" s="3" t="n"/>
-      <c r="K4" s="3" t="n"/>
-      <c r="L4" s="3" t="n"/>
-      <c r="M4" s="3" t="n"/>
-      <c r="N4" s="3" t="n"/>
-      <c r="O4" s="3" t="n"/>
-      <c r="P4" s="3" t="n"/>
-      <c r="Q4" s="3" t="n"/>
-      <c r="R4" s="3" t="n"/>
-      <c r="S4" s="3" t="n"/>
-      <c r="T4" s="4">
+      <c r="J4" s="4" t="n"/>
+      <c r="K4" s="4" t="n"/>
+      <c r="L4" s="4" t="n"/>
+      <c r="M4" s="4" t="n"/>
+      <c r="N4" s="4" t="n"/>
+      <c r="O4" s="4" t="n"/>
+      <c r="P4" s="4" t="n"/>
+      <c r="Q4" s="4" t="n"/>
+      <c r="R4" s="4" t="n"/>
+      <c r="S4" s="4" t="n"/>
+      <c r="T4" s="5">
         <f>SUM(J4:S4)</f>
         <v/>
       </c>
       <c r="U4">
-        <f>IF(COUNT(J4:S4)=0,"",IF(COUNT(J4:S4)&lt;10,"INCOMPLETE",IF(T4=$V$2,"OK","OFF BY "&amp;TEXT(T4-$V$2,"+0;-0"))))</f>
-        <v/>
+        <f>IF(COUNT(J4:S4)=0,"",IF(COUNT(J4:S4)&lt;10,"INCOMPLETE",IF(N(V4)=0,"",IF(T4=V4,"OK","OFF BY "&amp;TEXT(T4-V4,"+0;-0")))))</f>
+        <v/>
+      </c>
+      <c r="V4">
+        <f>IF(N($Y$2)+N($Y$3)=0,"",IF($I4=1,$Y$2,$Y$3))</f>
+        <v/>
+      </c>
+      <c r="X4" s="6" t="inlineStr">
+        <is>
+          <t>Blank = no target. Need not match; a shorter reach may earn more.</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -816,12 +846,12 @@
           <t>Light</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Earth</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Dark</t>
         </is>
@@ -829,22 +859,26 @@
       <c r="I5" t="n">
         <v>2</v>
       </c>
-      <c r="J5" s="3" t="n"/>
-      <c r="K5" s="3" t="n"/>
-      <c r="L5" s="3" t="n"/>
-      <c r="M5" s="3" t="n"/>
-      <c r="N5" s="3" t="n"/>
-      <c r="O5" s="3" t="n"/>
-      <c r="P5" s="3" t="n"/>
-      <c r="Q5" s="3" t="n"/>
-      <c r="R5" s="3" t="n"/>
-      <c r="S5" s="3" t="n"/>
-      <c r="T5" s="4">
+      <c r="J5" s="4" t="n"/>
+      <c r="K5" s="4" t="n"/>
+      <c r="L5" s="4" t="n"/>
+      <c r="M5" s="4" t="n"/>
+      <c r="N5" s="4" t="n"/>
+      <c r="O5" s="4" t="n"/>
+      <c r="P5" s="4" t="n"/>
+      <c r="Q5" s="4" t="n"/>
+      <c r="R5" s="4" t="n"/>
+      <c r="S5" s="4" t="n"/>
+      <c r="T5" s="5">
         <f>SUM(J5:S5)</f>
         <v/>
       </c>
       <c r="U5">
-        <f>IF(COUNT(J5:S5)=0,"",IF(COUNT(J5:S5)&lt;10,"INCOMPLETE",IF(T5=$V$2,"OK","OFF BY "&amp;TEXT(T5-$V$2,"+0;-0"))))</f>
+        <f>IF(COUNT(J5:S5)=0,"",IF(COUNT(J5:S5)&lt;10,"INCOMPLETE",IF(N(V5)=0,"",IF(T5=V5,"OK","OFF BY "&amp;TEXT(T5-V5,"+0;-0")))))</f>
+        <v/>
+      </c>
+      <c r="V5">
+        <f>IF(N($Y$2)+N($Y$3)=0,"",IF($I5=1,$Y$2,$Y$3))</f>
         <v/>
       </c>
     </row>
@@ -877,12 +911,12 @@
           <t>Water</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Earth</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>Fire</t>
         </is>
@@ -890,23 +924,32 @@
       <c r="I6" t="n">
         <v>2</v>
       </c>
-      <c r="J6" s="3" t="n"/>
-      <c r="K6" s="3" t="n"/>
-      <c r="L6" s="3" t="n"/>
-      <c r="M6" s="3" t="n"/>
-      <c r="N6" s="3" t="n"/>
-      <c r="O6" s="3" t="n"/>
-      <c r="P6" s="3" t="n"/>
-      <c r="Q6" s="3" t="n"/>
-      <c r="R6" s="3" t="n"/>
-      <c r="S6" s="3" t="n"/>
-      <c r="T6" s="4">
+      <c r="J6" s="4" t="n"/>
+      <c r="K6" s="4" t="n"/>
+      <c r="L6" s="4" t="n"/>
+      <c r="M6" s="4" t="n"/>
+      <c r="N6" s="4" t="n"/>
+      <c r="O6" s="4" t="n"/>
+      <c r="P6" s="4" t="n"/>
+      <c r="Q6" s="4" t="n"/>
+      <c r="R6" s="4" t="n"/>
+      <c r="S6" s="4" t="n"/>
+      <c r="T6" s="5">
         <f>SUM(J6:S6)</f>
         <v/>
       </c>
       <c r="U6">
-        <f>IF(COUNT(J6:S6)=0,"",IF(COUNT(J6:S6)&lt;10,"INCOMPLETE",IF(T6=$V$2,"OK","OFF BY "&amp;TEXT(T6-$V$2,"+0;-0"))))</f>
-        <v/>
+        <f>IF(COUNT(J6:S6)=0,"",IF(COUNT(J6:S6)&lt;10,"INCOMPLETE",IF(N(V6)=0,"",IF(T6=V6,"OK","OFF BY "&amp;TEXT(T6-V6,"+0;-0")))))</f>
+        <v/>
+      </c>
+      <c r="V6">
+        <f>IF(N($Y$2)+N($Y$3)=0,"",IF($I6=1,$Y$2,$Y$3))</f>
+        <v/>
+      </c>
+      <c r="X6" s="2" t="inlineStr">
+        <is>
+          <t>SPREAD</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -938,12 +981,12 @@
           <t>Dark</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Earth</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Light</t>
         </is>
@@ -951,23 +994,42 @@
       <c r="I7" t="n">
         <v>1</v>
       </c>
-      <c r="J7" s="3" t="n"/>
-      <c r="K7" s="3" t="n"/>
-      <c r="L7" s="3" t="n"/>
-      <c r="M7" s="3" t="n"/>
-      <c r="N7" s="3" t="n"/>
-      <c r="O7" s="3" t="n"/>
-      <c r="P7" s="3" t="n"/>
-      <c r="Q7" s="3" t="n"/>
-      <c r="R7" s="3" t="n"/>
-      <c r="S7" s="3" t="n"/>
-      <c r="T7" s="4">
+      <c r="J7" s="4" t="n"/>
+      <c r="K7" s="4" t="n"/>
+      <c r="L7" s="4" t="n"/>
+      <c r="M7" s="4" t="n"/>
+      <c r="N7" s="4" t="n"/>
+      <c r="O7" s="4" t="n"/>
+      <c r="P7" s="4" t="n"/>
+      <c r="Q7" s="4" t="n"/>
+      <c r="R7" s="4" t="n"/>
+      <c r="S7" s="4" t="n"/>
+      <c r="T7" s="5">
         <f>SUM(J7:S7)</f>
         <v/>
       </c>
       <c r="U7">
-        <f>IF(COUNT(J7:S7)=0,"",IF(COUNT(J7:S7)&lt;10,"INCOMPLETE",IF(T7=$V$2,"OK","OFF BY "&amp;TEXT(T7-$V$2,"+0;-0"))))</f>
-        <v/>
+        <f>IF(COUNT(J7:S7)=0,"",IF(COUNT(J7:S7)&lt;10,"INCOMPLETE",IF(N(V7)=0,"",IF(T7=V7,"OK","OFF BY "&amp;TEXT(T7-V7,"+0;-0")))))</f>
+        <v/>
+      </c>
+      <c r="V7">
+        <f>IF(N($Y$2)+N($Y$3)=0,"",IF($I7=1,$Y$2,$Y$3))</f>
+        <v/>
+      </c>
+      <c r="X7" s="5" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="Y7" s="5" t="inlineStr">
+        <is>
+          <t>Heroes</t>
+        </is>
+      </c>
+      <c r="Z7" s="5" t="inlineStr">
+        <is>
+          <t>Avg TOTAL</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -999,12 +1061,12 @@
           <t>Air</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Water</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>Earth</t>
         </is>
@@ -1012,22 +1074,39 @@
       <c r="I8" t="n">
         <v>1</v>
       </c>
-      <c r="J8" s="3" t="n"/>
-      <c r="K8" s="3" t="n"/>
-      <c r="L8" s="3" t="n"/>
-      <c r="M8" s="3" t="n"/>
-      <c r="N8" s="3" t="n"/>
-      <c r="O8" s="3" t="n"/>
-      <c r="P8" s="3" t="n"/>
-      <c r="Q8" s="3" t="n"/>
-      <c r="R8" s="3" t="n"/>
-      <c r="S8" s="3" t="n"/>
-      <c r="T8" s="4">
+      <c r="J8" s="4" t="n"/>
+      <c r="K8" s="4" t="n"/>
+      <c r="L8" s="4" t="n"/>
+      <c r="M8" s="4" t="n"/>
+      <c r="N8" s="4" t="n"/>
+      <c r="O8" s="4" t="n"/>
+      <c r="P8" s="4" t="n"/>
+      <c r="Q8" s="4" t="n"/>
+      <c r="R8" s="4" t="n"/>
+      <c r="S8" s="4" t="n"/>
+      <c r="T8" s="5">
         <f>SUM(J8:S8)</f>
         <v/>
       </c>
       <c r="U8">
-        <f>IF(COUNT(J8:S8)=0,"",IF(COUNT(J8:S8)&lt;10,"INCOMPLETE",IF(T8=$V$2,"OK","OFF BY "&amp;TEXT(T8-$V$2,"+0;-0"))))</f>
+        <f>IF(COUNT(J8:S8)=0,"",IF(COUNT(J8:S8)&lt;10,"INCOMPLETE",IF(N(V8)=0,"",IF(T8=V8,"OK","OFF BY "&amp;TEXT(T8-V8,"+0;-0")))))</f>
+        <v/>
+      </c>
+      <c r="V8">
+        <f>IF(N($Y$2)+N($Y$3)=0,"",IF($I8=1,$Y$2,$Y$3))</f>
+        <v/>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>Reach 1</t>
+        </is>
+      </c>
+      <c r="Y8">
+        <f>COUNTIF(I2:I28,1)</f>
+        <v/>
+      </c>
+      <c r="Z8">
+        <f>IFERROR(ROUND(AVERAGEIF(I2:I28,1,T2:T28),1),"")</f>
         <v/>
       </c>
     </row>
@@ -1060,12 +1139,12 @@
           <t>Light</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Water</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>Dark</t>
         </is>
@@ -1073,22 +1152,39 @@
       <c r="I9" t="n">
         <v>1</v>
       </c>
-      <c r="J9" s="3" t="n"/>
-      <c r="K9" s="3" t="n"/>
-      <c r="L9" s="3" t="n"/>
-      <c r="M9" s="3" t="n"/>
-      <c r="N9" s="3" t="n"/>
-      <c r="O9" s="3" t="n"/>
-      <c r="P9" s="3" t="n"/>
-      <c r="Q9" s="3" t="n"/>
-      <c r="R9" s="3" t="n"/>
-      <c r="S9" s="3" t="n"/>
-      <c r="T9" s="4">
+      <c r="J9" s="4" t="n"/>
+      <c r="K9" s="4" t="n"/>
+      <c r="L9" s="4" t="n"/>
+      <c r="M9" s="4" t="n"/>
+      <c r="N9" s="4" t="n"/>
+      <c r="O9" s="4" t="n"/>
+      <c r="P9" s="4" t="n"/>
+      <c r="Q9" s="4" t="n"/>
+      <c r="R9" s="4" t="n"/>
+      <c r="S9" s="4" t="n"/>
+      <c r="T9" s="5">
         <f>SUM(J9:S9)</f>
         <v/>
       </c>
       <c r="U9">
-        <f>IF(COUNT(J9:S9)=0,"",IF(COUNT(J9:S9)&lt;10,"INCOMPLETE",IF(T9=$V$2,"OK","OFF BY "&amp;TEXT(T9-$V$2,"+0;-0"))))</f>
+        <f>IF(COUNT(J9:S9)=0,"",IF(COUNT(J9:S9)&lt;10,"INCOMPLETE",IF(N(V9)=0,"",IF(T9=V9,"OK","OFF BY "&amp;TEXT(T9-V9,"+0;-0")))))</f>
+        <v/>
+      </c>
+      <c r="V9">
+        <f>IF(N($Y$2)+N($Y$3)=0,"",IF($I9=1,$Y$2,$Y$3))</f>
+        <v/>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>Reach 2</t>
+        </is>
+      </c>
+      <c r="Y9">
+        <f>COUNTIF(I2:I28,2)</f>
+        <v/>
+      </c>
+      <c r="Z9">
+        <f>IFERROR(ROUND(AVERAGEIF(I2:I28,2,T2:T28),1),"")</f>
         <v/>
       </c>
     </row>
@@ -1121,12 +1217,12 @@
           <t>Earth</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Water</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>Air</t>
         </is>
@@ -1134,22 +1230,39 @@
       <c r="I10" t="n">
         <v>2</v>
       </c>
-      <c r="J10" s="3" t="n"/>
-      <c r="K10" s="3" t="n"/>
-      <c r="L10" s="3" t="n"/>
-      <c r="M10" s="3" t="n"/>
-      <c r="N10" s="3" t="n"/>
-      <c r="O10" s="3" t="n"/>
-      <c r="P10" s="3" t="n"/>
-      <c r="Q10" s="3" t="n"/>
-      <c r="R10" s="3" t="n"/>
-      <c r="S10" s="3" t="n"/>
-      <c r="T10" s="4">
+      <c r="J10" s="4" t="n"/>
+      <c r="K10" s="4" t="n"/>
+      <c r="L10" s="4" t="n"/>
+      <c r="M10" s="4" t="n"/>
+      <c r="N10" s="4" t="n"/>
+      <c r="O10" s="4" t="n"/>
+      <c r="P10" s="4" t="n"/>
+      <c r="Q10" s="4" t="n"/>
+      <c r="R10" s="4" t="n"/>
+      <c r="S10" s="4" t="n"/>
+      <c r="T10" s="5">
         <f>SUM(J10:S10)</f>
         <v/>
       </c>
       <c r="U10">
-        <f>IF(COUNT(J10:S10)=0,"",IF(COUNT(J10:S10)&lt;10,"INCOMPLETE",IF(T10=$V$2,"OK","OFF BY "&amp;TEXT(T10-$V$2,"+0;-0"))))</f>
+        <f>IF(COUNT(J10:S10)=0,"",IF(COUNT(J10:S10)&lt;10,"INCOMPLETE",IF(N(V10)=0,"",IF(T10=V10,"OK","OFF BY "&amp;TEXT(T10-V10,"+0;-0")))))</f>
+        <v/>
+      </c>
+      <c r="V10">
+        <f>IF(N($Y$2)+N($Y$3)=0,"",IF($I10=1,$Y$2,$Y$3))</f>
+        <v/>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="Y10">
+        <f>COUNT(I2:I28)</f>
+        <v/>
+      </c>
+      <c r="Z10">
+        <f>IFERROR(ROUND(AVERAGE(T2:T28),1),"")</f>
         <v/>
       </c>
     </row>
@@ -1182,12 +1295,12 @@
           <t>Dark</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Fire</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>Light</t>
         </is>
@@ -1195,22 +1308,26 @@
       <c r="I11" t="n">
         <v>2</v>
       </c>
-      <c r="J11" s="3" t="n"/>
-      <c r="K11" s="3" t="n"/>
-      <c r="L11" s="3" t="n"/>
-      <c r="M11" s="3" t="n"/>
-      <c r="N11" s="3" t="n"/>
-      <c r="O11" s="3" t="n"/>
-      <c r="P11" s="3" t="n"/>
-      <c r="Q11" s="3" t="n"/>
-      <c r="R11" s="3" t="n"/>
-      <c r="S11" s="3" t="n"/>
-      <c r="T11" s="4">
+      <c r="J11" s="4" t="n"/>
+      <c r="K11" s="4" t="n"/>
+      <c r="L11" s="4" t="n"/>
+      <c r="M11" s="4" t="n"/>
+      <c r="N11" s="4" t="n"/>
+      <c r="O11" s="4" t="n"/>
+      <c r="P11" s="4" t="n"/>
+      <c r="Q11" s="4" t="n"/>
+      <c r="R11" s="4" t="n"/>
+      <c r="S11" s="4" t="n"/>
+      <c r="T11" s="5">
         <f>SUM(J11:S11)</f>
         <v/>
       </c>
       <c r="U11">
-        <f>IF(COUNT(J11:S11)=0,"",IF(COUNT(J11:S11)&lt;10,"INCOMPLETE",IF(T11=$V$2,"OK","OFF BY "&amp;TEXT(T11-$V$2,"+0;-0"))))</f>
+        <f>IF(COUNT(J11:S11)=0,"",IF(COUNT(J11:S11)&lt;10,"INCOMPLETE",IF(N(V11)=0,"",IF(T11=V11,"OK","OFF BY "&amp;TEXT(T11-V11,"+0;-0")))))</f>
+        <v/>
+      </c>
+      <c r="V11">
+        <f>IF(N($Y$2)+N($Y$3)=0,"",IF($I11=1,$Y$2,$Y$3))</f>
         <v/>
       </c>
     </row>
@@ -1243,12 +1360,12 @@
           <t>Earth</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>Fire</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>Air</t>
         </is>
@@ -1256,22 +1373,26 @@
       <c r="I12" t="n">
         <v>1</v>
       </c>
-      <c r="J12" s="3" t="n"/>
-      <c r="K12" s="3" t="n"/>
-      <c r="L12" s="3" t="n"/>
-      <c r="M12" s="3" t="n"/>
-      <c r="N12" s="3" t="n"/>
-      <c r="O12" s="3" t="n"/>
-      <c r="P12" s="3" t="n"/>
-      <c r="Q12" s="3" t="n"/>
-      <c r="R12" s="3" t="n"/>
-      <c r="S12" s="3" t="n"/>
-      <c r="T12" s="4">
+      <c r="J12" s="4" t="n"/>
+      <c r="K12" s="4" t="n"/>
+      <c r="L12" s="4" t="n"/>
+      <c r="M12" s="4" t="n"/>
+      <c r="N12" s="4" t="n"/>
+      <c r="O12" s="4" t="n"/>
+      <c r="P12" s="4" t="n"/>
+      <c r="Q12" s="4" t="n"/>
+      <c r="R12" s="4" t="n"/>
+      <c r="S12" s="4" t="n"/>
+      <c r="T12" s="5">
         <f>SUM(J12:S12)</f>
         <v/>
       </c>
       <c r="U12">
-        <f>IF(COUNT(J12:S12)=0,"",IF(COUNT(J12:S12)&lt;10,"INCOMPLETE",IF(T12=$V$2,"OK","OFF BY "&amp;TEXT(T12-$V$2,"+0;-0"))))</f>
+        <f>IF(COUNT(J12:S12)=0,"",IF(COUNT(J12:S12)&lt;10,"INCOMPLETE",IF(N(V12)=0,"",IF(T12=V12,"OK","OFF BY "&amp;TEXT(T12-V12,"+0;-0")))))</f>
+        <v/>
+      </c>
+      <c r="V12">
+        <f>IF(N($Y$2)+N($Y$3)=0,"",IF($I12=1,$Y$2,$Y$3))</f>
         <v/>
       </c>
     </row>
@@ -1304,12 +1425,12 @@
           <t>Air</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Fire</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>Earth</t>
         </is>
@@ -1317,22 +1438,26 @@
       <c r="I13" t="n">
         <v>2</v>
       </c>
-      <c r="J13" s="3" t="n"/>
-      <c r="K13" s="3" t="n"/>
-      <c r="L13" s="3" t="n"/>
-      <c r="M13" s="3" t="n"/>
-      <c r="N13" s="3" t="n"/>
-      <c r="O13" s="3" t="n"/>
-      <c r="P13" s="3" t="n"/>
-      <c r="Q13" s="3" t="n"/>
-      <c r="R13" s="3" t="n"/>
-      <c r="S13" s="3" t="n"/>
-      <c r="T13" s="4">
+      <c r="J13" s="4" t="n"/>
+      <c r="K13" s="4" t="n"/>
+      <c r="L13" s="4" t="n"/>
+      <c r="M13" s="4" t="n"/>
+      <c r="N13" s="4" t="n"/>
+      <c r="O13" s="4" t="n"/>
+      <c r="P13" s="4" t="n"/>
+      <c r="Q13" s="4" t="n"/>
+      <c r="R13" s="4" t="n"/>
+      <c r="S13" s="4" t="n"/>
+      <c r="T13" s="5">
         <f>SUM(J13:S13)</f>
         <v/>
       </c>
       <c r="U13">
-        <f>IF(COUNT(J13:S13)=0,"",IF(COUNT(J13:S13)&lt;10,"INCOMPLETE",IF(T13=$V$2,"OK","OFF BY "&amp;TEXT(T13-$V$2,"+0;-0"))))</f>
+        <f>IF(COUNT(J13:S13)=0,"",IF(COUNT(J13:S13)&lt;10,"INCOMPLETE",IF(N(V13)=0,"",IF(T13=V13,"OK","OFF BY "&amp;TEXT(T13-V13,"+0;-0")))))</f>
+        <v/>
+      </c>
+      <c r="V13">
+        <f>IF(N($Y$2)+N($Y$3)=0,"",IF($I13=1,$Y$2,$Y$3))</f>
         <v/>
       </c>
     </row>
@@ -1365,12 +1490,12 @@
           <t>Fire</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>Dark</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>Water</t>
         </is>
@@ -1378,22 +1503,26 @@
       <c r="I14" t="n">
         <v>1</v>
       </c>
-      <c r="J14" s="3" t="n"/>
-      <c r="K14" s="3" t="n"/>
-      <c r="L14" s="3" t="n"/>
-      <c r="M14" s="3" t="n"/>
-      <c r="N14" s="3" t="n"/>
-      <c r="O14" s="3" t="n"/>
-      <c r="P14" s="3" t="n"/>
-      <c r="Q14" s="3" t="n"/>
-      <c r="R14" s="3" t="n"/>
-      <c r="S14" s="3" t="n"/>
-      <c r="T14" s="4">
+      <c r="J14" s="4" t="n"/>
+      <c r="K14" s="4" t="n"/>
+      <c r="L14" s="4" t="n"/>
+      <c r="M14" s="4" t="n"/>
+      <c r="N14" s="4" t="n"/>
+      <c r="O14" s="4" t="n"/>
+      <c r="P14" s="4" t="n"/>
+      <c r="Q14" s="4" t="n"/>
+      <c r="R14" s="4" t="n"/>
+      <c r="S14" s="4" t="n"/>
+      <c r="T14" s="5">
         <f>SUM(J14:S14)</f>
         <v/>
       </c>
       <c r="U14">
-        <f>IF(COUNT(J14:S14)=0,"",IF(COUNT(J14:S14)&lt;10,"INCOMPLETE",IF(T14=$V$2,"OK","OFF BY "&amp;TEXT(T14-$V$2,"+0;-0"))))</f>
+        <f>IF(COUNT(J14:S14)=0,"",IF(COUNT(J14:S14)&lt;10,"INCOMPLETE",IF(N(V14)=0,"",IF(T14=V14,"OK","OFF BY "&amp;TEXT(T14-V14,"+0;-0")))))</f>
+        <v/>
+      </c>
+      <c r="V14">
+        <f>IF(N($Y$2)+N($Y$3)=0,"",IF($I14=1,$Y$2,$Y$3))</f>
         <v/>
       </c>
     </row>
@@ -1426,12 +1555,12 @@
           <t>Air</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>Dark</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr">
         <is>
           <t>Earth</t>
         </is>
@@ -1439,22 +1568,26 @@
       <c r="I15" t="n">
         <v>2</v>
       </c>
-      <c r="J15" s="3" t="n"/>
-      <c r="K15" s="3" t="n"/>
-      <c r="L15" s="3" t="n"/>
-      <c r="M15" s="3" t="n"/>
-      <c r="N15" s="3" t="n"/>
-      <c r="O15" s="3" t="n"/>
-      <c r="P15" s="3" t="n"/>
-      <c r="Q15" s="3" t="n"/>
-      <c r="R15" s="3" t="n"/>
-      <c r="S15" s="3" t="n"/>
-      <c r="T15" s="4">
+      <c r="J15" s="4" t="n"/>
+      <c r="K15" s="4" t="n"/>
+      <c r="L15" s="4" t="n"/>
+      <c r="M15" s="4" t="n"/>
+      <c r="N15" s="4" t="n"/>
+      <c r="O15" s="4" t="n"/>
+      <c r="P15" s="4" t="n"/>
+      <c r="Q15" s="4" t="n"/>
+      <c r="R15" s="4" t="n"/>
+      <c r="S15" s="4" t="n"/>
+      <c r="T15" s="5">
         <f>SUM(J15:S15)</f>
         <v/>
       </c>
       <c r="U15">
-        <f>IF(COUNT(J15:S15)=0,"",IF(COUNT(J15:S15)&lt;10,"INCOMPLETE",IF(T15=$V$2,"OK","OFF BY "&amp;TEXT(T15-$V$2,"+0;-0"))))</f>
+        <f>IF(COUNT(J15:S15)=0,"",IF(COUNT(J15:S15)&lt;10,"INCOMPLETE",IF(N(V15)=0,"",IF(T15=V15,"OK","OFF BY "&amp;TEXT(T15-V15,"+0;-0")))))</f>
+        <v/>
+      </c>
+      <c r="V15">
+        <f>IF(N($Y$2)+N($Y$3)=0,"",IF($I15=1,$Y$2,$Y$3))</f>
         <v/>
       </c>
     </row>
@@ -1487,12 +1620,12 @@
           <t>Water</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>Dark</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H16" s="3" t="inlineStr">
         <is>
           <t>Fire</t>
         </is>
@@ -1500,22 +1633,26 @@
       <c r="I16" t="n">
         <v>2</v>
       </c>
-      <c r="J16" s="3" t="n"/>
-      <c r="K16" s="3" t="n"/>
-      <c r="L16" s="3" t="n"/>
-      <c r="M16" s="3" t="n"/>
-      <c r="N16" s="3" t="n"/>
-      <c r="O16" s="3" t="n"/>
-      <c r="P16" s="3" t="n"/>
-      <c r="Q16" s="3" t="n"/>
-      <c r="R16" s="3" t="n"/>
-      <c r="S16" s="3" t="n"/>
-      <c r="T16" s="4">
+      <c r="J16" s="4" t="n"/>
+      <c r="K16" s="4" t="n"/>
+      <c r="L16" s="4" t="n"/>
+      <c r="M16" s="4" t="n"/>
+      <c r="N16" s="4" t="n"/>
+      <c r="O16" s="4" t="n"/>
+      <c r="P16" s="4" t="n"/>
+      <c r="Q16" s="4" t="n"/>
+      <c r="R16" s="4" t="n"/>
+      <c r="S16" s="4" t="n"/>
+      <c r="T16" s="5">
         <f>SUM(J16:S16)</f>
         <v/>
       </c>
       <c r="U16">
-        <f>IF(COUNT(J16:S16)=0,"",IF(COUNT(J16:S16)&lt;10,"INCOMPLETE",IF(T16=$V$2,"OK","OFF BY "&amp;TEXT(T16-$V$2,"+0;-0"))))</f>
+        <f>IF(COUNT(J16:S16)=0,"",IF(COUNT(J16:S16)&lt;10,"INCOMPLETE",IF(N(V16)=0,"",IF(T16=V16,"OK","OFF BY "&amp;TEXT(T16-V16,"+0;-0")))))</f>
+        <v/>
+      </c>
+      <c r="V16">
+        <f>IF(N($Y$2)+N($Y$3)=0,"",IF($I16=1,$Y$2,$Y$3))</f>
         <v/>
       </c>
     </row>
@@ -1548,12 +1685,12 @@
           <t>Water</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>Light</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>Fire</t>
         </is>
@@ -1561,22 +1698,26 @@
       <c r="I17" t="n">
         <v>2</v>
       </c>
-      <c r="J17" s="3" t="n"/>
-      <c r="K17" s="3" t="n"/>
-      <c r="L17" s="3" t="n"/>
-      <c r="M17" s="3" t="n"/>
-      <c r="N17" s="3" t="n"/>
-      <c r="O17" s="3" t="n"/>
-      <c r="P17" s="3" t="n"/>
-      <c r="Q17" s="3" t="n"/>
-      <c r="R17" s="3" t="n"/>
-      <c r="S17" s="3" t="n"/>
-      <c r="T17" s="4">
+      <c r="J17" s="4" t="n"/>
+      <c r="K17" s="4" t="n"/>
+      <c r="L17" s="4" t="n"/>
+      <c r="M17" s="4" t="n"/>
+      <c r="N17" s="4" t="n"/>
+      <c r="O17" s="4" t="n"/>
+      <c r="P17" s="4" t="n"/>
+      <c r="Q17" s="4" t="n"/>
+      <c r="R17" s="4" t="n"/>
+      <c r="S17" s="4" t="n"/>
+      <c r="T17" s="5">
         <f>SUM(J17:S17)</f>
         <v/>
       </c>
       <c r="U17">
-        <f>IF(COUNT(J17:S17)=0,"",IF(COUNT(J17:S17)&lt;10,"INCOMPLETE",IF(T17=$V$2,"OK","OFF BY "&amp;TEXT(T17-$V$2,"+0;-0"))))</f>
+        <f>IF(COUNT(J17:S17)=0,"",IF(COUNT(J17:S17)&lt;10,"INCOMPLETE",IF(N(V17)=0,"",IF(T17=V17,"OK","OFF BY "&amp;TEXT(T17-V17,"+0;-0")))))</f>
+        <v/>
+      </c>
+      <c r="V17">
+        <f>IF(N($Y$2)+N($Y$3)=0,"",IF($I17=1,$Y$2,$Y$3))</f>
         <v/>
       </c>
     </row>
@@ -1609,12 +1750,12 @@
           <t>Fire</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>Light</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>Water</t>
         </is>
@@ -1622,22 +1763,26 @@
       <c r="I18" t="n">
         <v>1</v>
       </c>
-      <c r="J18" s="3" t="n"/>
-      <c r="K18" s="3" t="n"/>
-      <c r="L18" s="3" t="n"/>
-      <c r="M18" s="3" t="n"/>
-      <c r="N18" s="3" t="n"/>
-      <c r="O18" s="3" t="n"/>
-      <c r="P18" s="3" t="n"/>
-      <c r="Q18" s="3" t="n"/>
-      <c r="R18" s="3" t="n"/>
-      <c r="S18" s="3" t="n"/>
-      <c r="T18" s="4">
+      <c r="J18" s="4" t="n"/>
+      <c r="K18" s="4" t="n"/>
+      <c r="L18" s="4" t="n"/>
+      <c r="M18" s="4" t="n"/>
+      <c r="N18" s="4" t="n"/>
+      <c r="O18" s="4" t="n"/>
+      <c r="P18" s="4" t="n"/>
+      <c r="Q18" s="4" t="n"/>
+      <c r="R18" s="4" t="n"/>
+      <c r="S18" s="4" t="n"/>
+      <c r="T18" s="5">
         <f>SUM(J18:S18)</f>
         <v/>
       </c>
       <c r="U18">
-        <f>IF(COUNT(J18:S18)=0,"",IF(COUNT(J18:S18)&lt;10,"INCOMPLETE",IF(T18=$V$2,"OK","OFF BY "&amp;TEXT(T18-$V$2,"+0;-0"))))</f>
+        <f>IF(COUNT(J18:S18)=0,"",IF(COUNT(J18:S18)&lt;10,"INCOMPLETE",IF(N(V18)=0,"",IF(T18=V18,"OK","OFF BY "&amp;TEXT(T18-V18,"+0;-0")))))</f>
+        <v/>
+      </c>
+      <c r="V18">
+        <f>IF(N($Y$2)+N($Y$3)=0,"",IF($I18=1,$Y$2,$Y$3))</f>
         <v/>
       </c>
     </row>
@@ -1670,12 +1815,12 @@
           <t>Earth</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>Light</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr">
         <is>
           <t>Air</t>
         </is>
@@ -1683,22 +1828,26 @@
       <c r="I19" t="n">
         <v>2</v>
       </c>
-      <c r="J19" s="3" t="n"/>
-      <c r="K19" s="3" t="n"/>
-      <c r="L19" s="3" t="n"/>
-      <c r="M19" s="3" t="n"/>
-      <c r="N19" s="3" t="n"/>
-      <c r="O19" s="3" t="n"/>
-      <c r="P19" s="3" t="n"/>
-      <c r="Q19" s="3" t="n"/>
-      <c r="R19" s="3" t="n"/>
-      <c r="S19" s="3" t="n"/>
-      <c r="T19" s="4">
+      <c r="J19" s="4" t="n"/>
+      <c r="K19" s="4" t="n"/>
+      <c r="L19" s="4" t="n"/>
+      <c r="M19" s="4" t="n"/>
+      <c r="N19" s="4" t="n"/>
+      <c r="O19" s="4" t="n"/>
+      <c r="P19" s="4" t="n"/>
+      <c r="Q19" s="4" t="n"/>
+      <c r="R19" s="4" t="n"/>
+      <c r="S19" s="4" t="n"/>
+      <c r="T19" s="5">
         <f>SUM(J19:S19)</f>
         <v/>
       </c>
       <c r="U19">
-        <f>IF(COUNT(J19:S19)=0,"",IF(COUNT(J19:S19)&lt;10,"INCOMPLETE",IF(T19=$V$2,"OK","OFF BY "&amp;TEXT(T19-$V$2,"+0;-0"))))</f>
+        <f>IF(COUNT(J19:S19)=0,"",IF(COUNT(J19:S19)&lt;10,"INCOMPLETE",IF(N(V19)=0,"",IF(T19=V19,"OK","OFF BY "&amp;TEXT(T19-V19,"+0;-0")))))</f>
+        <v/>
+      </c>
+      <c r="V19">
+        <f>IF(N($Y$2)+N($Y$3)=0,"",IF($I19=1,$Y$2,$Y$3))</f>
         <v/>
       </c>
     </row>
@@ -1731,12 +1880,12 @@
           <t>Light</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>Crush</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H20" s="3" t="inlineStr">
         <is>
           <t>Dark</t>
         </is>
@@ -1744,22 +1893,26 @@
       <c r="I20" t="n">
         <v>1</v>
       </c>
-      <c r="J20" s="3" t="n"/>
-      <c r="K20" s="3" t="n"/>
-      <c r="L20" s="3" t="n"/>
-      <c r="M20" s="3" t="n"/>
-      <c r="N20" s="3" t="n"/>
-      <c r="O20" s="3" t="n"/>
-      <c r="P20" s="3" t="n"/>
-      <c r="Q20" s="3" t="n"/>
-      <c r="R20" s="3" t="n"/>
-      <c r="S20" s="3" t="n"/>
-      <c r="T20" s="4">
+      <c r="J20" s="4" t="n"/>
+      <c r="K20" s="4" t="n"/>
+      <c r="L20" s="4" t="n"/>
+      <c r="M20" s="4" t="n"/>
+      <c r="N20" s="4" t="n"/>
+      <c r="O20" s="4" t="n"/>
+      <c r="P20" s="4" t="n"/>
+      <c r="Q20" s="4" t="n"/>
+      <c r="R20" s="4" t="n"/>
+      <c r="S20" s="4" t="n"/>
+      <c r="T20" s="5">
         <f>SUM(J20:S20)</f>
         <v/>
       </c>
       <c r="U20">
-        <f>IF(COUNT(J20:S20)=0,"",IF(COUNT(J20:S20)&lt;10,"INCOMPLETE",IF(T20=$V$2,"OK","OFF BY "&amp;TEXT(T20-$V$2,"+0;-0"))))</f>
+        <f>IF(COUNT(J20:S20)=0,"",IF(COUNT(J20:S20)&lt;10,"INCOMPLETE",IF(N(V20)=0,"",IF(T20=V20,"OK","OFF BY "&amp;TEXT(T20-V20,"+0;-0")))))</f>
+        <v/>
+      </c>
+      <c r="V20">
+        <f>IF(N($Y$2)+N($Y$3)=0,"",IF($I20=1,$Y$2,$Y$3))</f>
         <v/>
       </c>
     </row>
@@ -1792,12 +1945,12 @@
           <t>Water</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>Crush</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>Fire</t>
         </is>
@@ -1805,22 +1958,26 @@
       <c r="I21" t="n">
         <v>1</v>
       </c>
-      <c r="J21" s="3" t="n"/>
-      <c r="K21" s="3" t="n"/>
-      <c r="L21" s="3" t="n"/>
-      <c r="M21" s="3" t="n"/>
-      <c r="N21" s="3" t="n"/>
-      <c r="O21" s="3" t="n"/>
-      <c r="P21" s="3" t="n"/>
-      <c r="Q21" s="3" t="n"/>
-      <c r="R21" s="3" t="n"/>
-      <c r="S21" s="3" t="n"/>
-      <c r="T21" s="4">
+      <c r="J21" s="4" t="n"/>
+      <c r="K21" s="4" t="n"/>
+      <c r="L21" s="4" t="n"/>
+      <c r="M21" s="4" t="n"/>
+      <c r="N21" s="4" t="n"/>
+      <c r="O21" s="4" t="n"/>
+      <c r="P21" s="4" t="n"/>
+      <c r="Q21" s="4" t="n"/>
+      <c r="R21" s="4" t="n"/>
+      <c r="S21" s="4" t="n"/>
+      <c r="T21" s="5">
         <f>SUM(J21:S21)</f>
         <v/>
       </c>
       <c r="U21">
-        <f>IF(COUNT(J21:S21)=0,"",IF(COUNT(J21:S21)&lt;10,"INCOMPLETE",IF(T21=$V$2,"OK","OFF BY "&amp;TEXT(T21-$V$2,"+0;-0"))))</f>
+        <f>IF(COUNT(J21:S21)=0,"",IF(COUNT(J21:S21)&lt;10,"INCOMPLETE",IF(N(V21)=0,"",IF(T21=V21,"OK","OFF BY "&amp;TEXT(T21-V21,"+0;-0")))))</f>
+        <v/>
+      </c>
+      <c r="V21">
+        <f>IF(N($Y$2)+N($Y$3)=0,"",IF($I21=1,$Y$2,$Y$3))</f>
         <v/>
       </c>
     </row>
@@ -1853,12 +2010,12 @@
           <t>Dark</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>Crush</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="H22" s="3" t="inlineStr">
         <is>
           <t>Light</t>
         </is>
@@ -1866,22 +2023,26 @@
       <c r="I22" t="n">
         <v>2</v>
       </c>
-      <c r="J22" s="3" t="n"/>
-      <c r="K22" s="3" t="n"/>
-      <c r="L22" s="3" t="n"/>
-      <c r="M22" s="3" t="n"/>
-      <c r="N22" s="3" t="n"/>
-      <c r="O22" s="3" t="n"/>
-      <c r="P22" s="3" t="n"/>
-      <c r="Q22" s="3" t="n"/>
-      <c r="R22" s="3" t="n"/>
-      <c r="S22" s="3" t="n"/>
-      <c r="T22" s="4">
+      <c r="J22" s="4" t="n"/>
+      <c r="K22" s="4" t="n"/>
+      <c r="L22" s="4" t="n"/>
+      <c r="M22" s="4" t="n"/>
+      <c r="N22" s="4" t="n"/>
+      <c r="O22" s="4" t="n"/>
+      <c r="P22" s="4" t="n"/>
+      <c r="Q22" s="4" t="n"/>
+      <c r="R22" s="4" t="n"/>
+      <c r="S22" s="4" t="n"/>
+      <c r="T22" s="5">
         <f>SUM(J22:S22)</f>
         <v/>
       </c>
       <c r="U22">
-        <f>IF(COUNT(J22:S22)=0,"",IF(COUNT(J22:S22)&lt;10,"INCOMPLETE",IF(T22=$V$2,"OK","OFF BY "&amp;TEXT(T22-$V$2,"+0;-0"))))</f>
+        <f>IF(COUNT(J22:S22)=0,"",IF(COUNT(J22:S22)&lt;10,"INCOMPLETE",IF(N(V22)=0,"",IF(T22=V22,"OK","OFF BY "&amp;TEXT(T22-V22,"+0;-0")))))</f>
+        <v/>
+      </c>
+      <c r="V22">
+        <f>IF(N($Y$2)+N($Y$3)=0,"",IF($I22=1,$Y$2,$Y$3))</f>
         <v/>
       </c>
     </row>
@@ -1914,12 +2075,12 @@
           <t>Air</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>Slash</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr">
         <is>
           <t>Earth</t>
         </is>
@@ -1927,22 +2088,26 @@
       <c r="I23" t="n">
         <v>2</v>
       </c>
-      <c r="J23" s="3" t="n"/>
-      <c r="K23" s="3" t="n"/>
-      <c r="L23" s="3" t="n"/>
-      <c r="M23" s="3" t="n"/>
-      <c r="N23" s="3" t="n"/>
-      <c r="O23" s="3" t="n"/>
-      <c r="P23" s="3" t="n"/>
-      <c r="Q23" s="3" t="n"/>
-      <c r="R23" s="3" t="n"/>
-      <c r="S23" s="3" t="n"/>
-      <c r="T23" s="4">
+      <c r="J23" s="4" t="n"/>
+      <c r="K23" s="4" t="n"/>
+      <c r="L23" s="4" t="n"/>
+      <c r="M23" s="4" t="n"/>
+      <c r="N23" s="4" t="n"/>
+      <c r="O23" s="4" t="n"/>
+      <c r="P23" s="4" t="n"/>
+      <c r="Q23" s="4" t="n"/>
+      <c r="R23" s="4" t="n"/>
+      <c r="S23" s="4" t="n"/>
+      <c r="T23" s="5">
         <f>SUM(J23:S23)</f>
         <v/>
       </c>
       <c r="U23">
-        <f>IF(COUNT(J23:S23)=0,"",IF(COUNT(J23:S23)&lt;10,"INCOMPLETE",IF(T23=$V$2,"OK","OFF BY "&amp;TEXT(T23-$V$2,"+0;-0"))))</f>
+        <f>IF(COUNT(J23:S23)=0,"",IF(COUNT(J23:S23)&lt;10,"INCOMPLETE",IF(N(V23)=0,"",IF(T23=V23,"OK","OFF BY "&amp;TEXT(T23-V23,"+0;-0")))))</f>
+        <v/>
+      </c>
+      <c r="V23">
+        <f>IF(N($Y$2)+N($Y$3)=0,"",IF($I23=1,$Y$2,$Y$3))</f>
         <v/>
       </c>
     </row>
@@ -1975,12 +2140,12 @@
           <t>Dark</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G24" s="3" t="inlineStr">
         <is>
           <t>Slash</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="H24" s="3" t="inlineStr">
         <is>
           <t>Light</t>
         </is>
@@ -1988,22 +2153,26 @@
       <c r="I24" t="n">
         <v>1</v>
       </c>
-      <c r="J24" s="3" t="n"/>
-      <c r="K24" s="3" t="n"/>
-      <c r="L24" s="3" t="n"/>
-      <c r="M24" s="3" t="n"/>
-      <c r="N24" s="3" t="n"/>
-      <c r="O24" s="3" t="n"/>
-      <c r="P24" s="3" t="n"/>
-      <c r="Q24" s="3" t="n"/>
-      <c r="R24" s="3" t="n"/>
-      <c r="S24" s="3" t="n"/>
-      <c r="T24" s="4">
+      <c r="J24" s="4" t="n"/>
+      <c r="K24" s="4" t="n"/>
+      <c r="L24" s="4" t="n"/>
+      <c r="M24" s="4" t="n"/>
+      <c r="N24" s="4" t="n"/>
+      <c r="O24" s="4" t="n"/>
+      <c r="P24" s="4" t="n"/>
+      <c r="Q24" s="4" t="n"/>
+      <c r="R24" s="4" t="n"/>
+      <c r="S24" s="4" t="n"/>
+      <c r="T24" s="5">
         <f>SUM(J24:S24)</f>
         <v/>
       </c>
       <c r="U24">
-        <f>IF(COUNT(J24:S24)=0,"",IF(COUNT(J24:S24)&lt;10,"INCOMPLETE",IF(T24=$V$2,"OK","OFF BY "&amp;TEXT(T24-$V$2,"+0;-0"))))</f>
+        <f>IF(COUNT(J24:S24)=0,"",IF(COUNT(J24:S24)&lt;10,"INCOMPLETE",IF(N(V24)=0,"",IF(T24=V24,"OK","OFF BY "&amp;TEXT(T24-V24,"+0;-0")))))</f>
+        <v/>
+      </c>
+      <c r="V24">
+        <f>IF(N($Y$2)+N($Y$3)=0,"",IF($I24=1,$Y$2,$Y$3))</f>
         <v/>
       </c>
     </row>
@@ -2036,12 +2205,12 @@
           <t>Light</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>Slash</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="H25" s="3" t="inlineStr">
         <is>
           <t>Dark</t>
         </is>
@@ -2049,22 +2218,26 @@
       <c r="I25" t="n">
         <v>2</v>
       </c>
-      <c r="J25" s="3" t="n"/>
-      <c r="K25" s="3" t="n"/>
-      <c r="L25" s="3" t="n"/>
-      <c r="M25" s="3" t="n"/>
-      <c r="N25" s="3" t="n"/>
-      <c r="O25" s="3" t="n"/>
-      <c r="P25" s="3" t="n"/>
-      <c r="Q25" s="3" t="n"/>
-      <c r="R25" s="3" t="n"/>
-      <c r="S25" s="3" t="n"/>
-      <c r="T25" s="4">
+      <c r="J25" s="4" t="n"/>
+      <c r="K25" s="4" t="n"/>
+      <c r="L25" s="4" t="n"/>
+      <c r="M25" s="4" t="n"/>
+      <c r="N25" s="4" t="n"/>
+      <c r="O25" s="4" t="n"/>
+      <c r="P25" s="4" t="n"/>
+      <c r="Q25" s="4" t="n"/>
+      <c r="R25" s="4" t="n"/>
+      <c r="S25" s="4" t="n"/>
+      <c r="T25" s="5">
         <f>SUM(J25:S25)</f>
         <v/>
       </c>
       <c r="U25">
-        <f>IF(COUNT(J25:S25)=0,"",IF(COUNT(J25:S25)&lt;10,"INCOMPLETE",IF(T25=$V$2,"OK","OFF BY "&amp;TEXT(T25-$V$2,"+0;-0"))))</f>
+        <f>IF(COUNT(J25:S25)=0,"",IF(COUNT(J25:S25)&lt;10,"INCOMPLETE",IF(N(V25)=0,"",IF(T25=V25,"OK","OFF BY "&amp;TEXT(T25-V25,"+0;-0")))))</f>
+        <v/>
+      </c>
+      <c r="V25">
+        <f>IF(N($Y$2)+N($Y$3)=0,"",IF($I25=1,$Y$2,$Y$3))</f>
         <v/>
       </c>
     </row>
@@ -2097,12 +2270,12 @@
           <t>Light</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>Pierce</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H26" s="3" t="inlineStr">
         <is>
           <t>Dark</t>
         </is>
@@ -2110,22 +2283,26 @@
       <c r="I26" t="n">
         <v>1</v>
       </c>
-      <c r="J26" s="3" t="n"/>
-      <c r="K26" s="3" t="n"/>
-      <c r="L26" s="3" t="n"/>
-      <c r="M26" s="3" t="n"/>
-      <c r="N26" s="3" t="n"/>
-      <c r="O26" s="3" t="n"/>
-      <c r="P26" s="3" t="n"/>
-      <c r="Q26" s="3" t="n"/>
-      <c r="R26" s="3" t="n"/>
-      <c r="S26" s="3" t="n"/>
-      <c r="T26" s="4">
+      <c r="J26" s="4" t="n"/>
+      <c r="K26" s="4" t="n"/>
+      <c r="L26" s="4" t="n"/>
+      <c r="M26" s="4" t="n"/>
+      <c r="N26" s="4" t="n"/>
+      <c r="O26" s="4" t="n"/>
+      <c r="P26" s="4" t="n"/>
+      <c r="Q26" s="4" t="n"/>
+      <c r="R26" s="4" t="n"/>
+      <c r="S26" s="4" t="n"/>
+      <c r="T26" s="5">
         <f>SUM(J26:S26)</f>
         <v/>
       </c>
       <c r="U26">
-        <f>IF(COUNT(J26:S26)=0,"",IF(COUNT(J26:S26)&lt;10,"INCOMPLETE",IF(T26=$V$2,"OK","OFF BY "&amp;TEXT(T26-$V$2,"+0;-0"))))</f>
+        <f>IF(COUNT(J26:S26)=0,"",IF(COUNT(J26:S26)&lt;10,"INCOMPLETE",IF(N(V26)=0,"",IF(T26=V26,"OK","OFF BY "&amp;TEXT(T26-V26,"+0;-0")))))</f>
+        <v/>
+      </c>
+      <c r="V26">
+        <f>IF(N($Y$2)+N($Y$3)=0,"",IF($I26=1,$Y$2,$Y$3))</f>
         <v/>
       </c>
     </row>
@@ -2158,12 +2335,12 @@
           <t>Dark</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>Pierce</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr">
         <is>
           <t>Light</t>
         </is>
@@ -2171,22 +2348,26 @@
       <c r="I27" t="n">
         <v>1</v>
       </c>
-      <c r="J27" s="3" t="n"/>
-      <c r="K27" s="3" t="n"/>
-      <c r="L27" s="3" t="n"/>
-      <c r="M27" s="3" t="n"/>
-      <c r="N27" s="3" t="n"/>
-      <c r="O27" s="3" t="n"/>
-      <c r="P27" s="3" t="n"/>
-      <c r="Q27" s="3" t="n"/>
-      <c r="R27" s="3" t="n"/>
-      <c r="S27" s="3" t="n"/>
-      <c r="T27" s="4">
+      <c r="J27" s="4" t="n"/>
+      <c r="K27" s="4" t="n"/>
+      <c r="L27" s="4" t="n"/>
+      <c r="M27" s="4" t="n"/>
+      <c r="N27" s="4" t="n"/>
+      <c r="O27" s="4" t="n"/>
+      <c r="P27" s="4" t="n"/>
+      <c r="Q27" s="4" t="n"/>
+      <c r="R27" s="4" t="n"/>
+      <c r="S27" s="4" t="n"/>
+      <c r="T27" s="5">
         <f>SUM(J27:S27)</f>
         <v/>
       </c>
       <c r="U27">
-        <f>IF(COUNT(J27:S27)=0,"",IF(COUNT(J27:S27)&lt;10,"INCOMPLETE",IF(T27=$V$2,"OK","OFF BY "&amp;TEXT(T27-$V$2,"+0;-0"))))</f>
+        <f>IF(COUNT(J27:S27)=0,"",IF(COUNT(J27:S27)&lt;10,"INCOMPLETE",IF(N(V27)=0,"",IF(T27=V27,"OK","OFF BY "&amp;TEXT(T27-V27,"+0;-0")))))</f>
+        <v/>
+      </c>
+      <c r="V27">
+        <f>IF(N($Y$2)+N($Y$3)=0,"",IF($I27=1,$Y$2,$Y$3))</f>
         <v/>
       </c>
     </row>
@@ -2219,12 +2400,12 @@
           <t>Earth</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G28" s="3" t="inlineStr">
         <is>
           <t>Pierce</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="H28" s="3" t="inlineStr">
         <is>
           <t>Air</t>
         </is>
@@ -2232,29 +2413,33 @@
       <c r="I28" t="n">
         <v>2</v>
       </c>
-      <c r="J28" s="3" t="n"/>
-      <c r="K28" s="3" t="n"/>
-      <c r="L28" s="3" t="n"/>
-      <c r="M28" s="3" t="n"/>
-      <c r="N28" s="3" t="n"/>
-      <c r="O28" s="3" t="n"/>
-      <c r="P28" s="3" t="n"/>
-      <c r="Q28" s="3" t="n"/>
-      <c r="R28" s="3" t="n"/>
-      <c r="S28" s="3" t="n"/>
-      <c r="T28" s="4">
+      <c r="J28" s="4" t="n"/>
+      <c r="K28" s="4" t="n"/>
+      <c r="L28" s="4" t="n"/>
+      <c r="M28" s="4" t="n"/>
+      <c r="N28" s="4" t="n"/>
+      <c r="O28" s="4" t="n"/>
+      <c r="P28" s="4" t="n"/>
+      <c r="Q28" s="4" t="n"/>
+      <c r="R28" s="4" t="n"/>
+      <c r="S28" s="4" t="n"/>
+      <c r="T28" s="5">
         <f>SUM(J28:S28)</f>
         <v/>
       </c>
       <c r="U28">
-        <f>IF(COUNT(J28:S28)=0,"",IF(COUNT(J28:S28)&lt;10,"INCOMPLETE",IF(T28=$V$2,"OK","OFF BY "&amp;TEXT(T28-$V$2,"+0;-0"))))</f>
+        <f>IF(COUNT(J28:S28)=0,"",IF(COUNT(J28:S28)&lt;10,"INCOMPLETE",IF(N(V28)=0,"",IF(T28=V28,"OK","OFF BY "&amp;TEXT(T28-V28,"+0;-0")))))</f>
+        <v/>
+      </c>
+      <c r="V28">
+        <f>IF(N($Y$2)+N($Y$3)=0,"",IF($I28=1,$Y$2,$Y$3))</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:V28"/>
   <dataValidations count="1">
-    <dataValidation sqref="J2:S28" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Out of range" error="Base stats are whole numbers from 1 to 50." promptTitle="Base stat" prompt="1-50. All ten must sum to the budget in V2." type="whole" operator="between">
+    <dataValidation sqref="J2:S28" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Outside the base range" error="Base stats are normally 1-50. Continue anyway?" promptTitle="Base stat" prompt="Normally 1-50. Totals are targets, not caps." type="whole" errorStyle="warning" operator="between">
       <formula1>1</formula1>
       <formula2>50</formula2>
     </dataValidation>
@@ -2269,7 +2454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2277,148 +2462,224 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>LMNTLZ — hero base stats</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Budget</t>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Targets</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>All ten base stats must sum to 250, identical for every hero.</t>
+          <t>Nothing here is capped. A target total is a guide you set, not a</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr"/>
+      <c r="A4" s="5" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Change it in one place: cell V2 of the Hero Stats sheet.</t>
+          <t>limit, and totals need not match across heroes.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Set Y2 (reach 1) and Y3 (reach 2) on the Hero Stats sheet and every</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>row's TARGET follows. A shorter-reach hero may be given the richer</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>budget — that is the point of splitting the target by reach.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Leave both blank and CHECK simply stays quiet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>For a one-off hero, overwrite that row's TARGET cell with a number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Base range</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Each base stat is a whole number from 1 to 50.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Hard cap</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>100 per stat after future growth. Growth is not designed yet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Each base stat is normally 1-50. Outside that you get a</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>warning you can dismiss, not a block.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Later ceiling</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>100 per stat once growth exists. Growth is not designed yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>CHECK column</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Blank until you start; INCOMPLETE until all ten are filled;</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr"/>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>then OK, or "OFF BY +n / -n" against the budget.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>then quiet if no target is set, else OK or "OFF BY +n / -n".</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>SPREAD block</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>X6:Z10 on the Hero Stats sheet — live hero counts and average</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>totals per reach group, so the reach/budget trade stays visible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Derived</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Bane and Fault are computed from Primary and Secondary and must</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr"/>
-      <c r="B11" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
         <is>
           <t>never be hand-edited. Bane = counter(Primary), Fault = counter(Secondary).</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr"/>
-      <c r="B12" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
         <is>
           <t>counter: Earth&lt;-&gt;Air, Fire&lt;-&gt;Water, Light&lt;-&gt;Dark, Crush&gt;Slash&gt;Pierce&gt;Crush.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="5" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Reach</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Proposed only — not settled, and NOT part of the stat budget.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr"/>
-      <c r="B15" t="inlineStr">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Proposed only — not settled, and NOT one of the ten stats.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
         <is>
           <t>It is positional: never scales, never enters a damage formula.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr"/>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>It does drive the TARGET column, which is a budgeting choice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>Regenerating</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>tools/build-hero-stats.py rebuilds this file and OVERWRITES it.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr"/>
-      <c r="B18" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
         <is>
           <t>Do not run it once real stat values have been entered.</t>
         </is>

</xml_diff>

<commit_message>
Add a Powers sheet: 27 heroes x 6 powers, named
Three tiers of sharing, generated from the type data already in the
workbook rather than typed per hero:

  0,1,2  shared by primary type -- 9 Houses x 3 = 27 names. Rank 0 is the
         auto-skill: the default attack, no cooldown, so a hero is never
         idle waiting on a timed power.
  3      shared by secondary type -- only 6 names, because melee always
         takes an arcane secondary, so no melee type appears here.
  4,5    unique per hero -- 54 names drawn from each concept and epithet.

87 distinct names across 162 cells, no collisions, no blanks. Voice
follows the House descriptions in LORE-and-flavor.md.

Names only -- effects, costs and cooldowns are not designed. Sharing tiers
are colour-coded so the structure reads at a glance, with a legend beside
the table. Hero Stats is untouched.
</commit_message>
<xml_diff>
--- a/resources/characters/hero-stats.xlsx
+++ b/resources/characters/hero-stats.xlsx
@@ -4,10 +4,12 @@
   <workbookPr/>
   <sheets>
     <sheet name="Hero Stats" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Rules" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Powers" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Rules" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hero Stats'!$A$1:$W$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Powers'!$A$1:$J$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -16,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -65,8 +67,18 @@
       <sz val="9"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFF4EFE4"/>
+    </font>
+    <font>
+      <i val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -91,6 +103,31 @@
         <bgColor rgb="FFFFFDF5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF241F38"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE6EEE2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEFF4EC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F0F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFDF5"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border/>
@@ -104,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -129,6 +166,15 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6953,6 +6999,1491 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" style="13" min="1" max="1"/>
+    <col width="20" customWidth="1" style="13" min="2" max="2"/>
+    <col width="11" customWidth="1" style="13" min="3" max="3"/>
+    <col width="12" customWidth="1" style="13" min="4" max="4"/>
+    <col width="22" customWidth="1" style="13" min="5" max="5"/>
+    <col width="22" customWidth="1" style="13" min="6" max="6"/>
+    <col width="26" customWidth="1" style="13" min="7" max="7"/>
+    <col width="26" customWidth="1" style="13" min="8" max="8"/>
+    <col width="26" customWidth="1" style="13" min="9" max="9"/>
+    <col width="28" customWidth="1" style="13" min="10" max="10"/>
+    <col width="66" customWidth="1" style="13" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1" s="13">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="14" t="inlineStr">
+        <is>
+          <t>Hero</t>
+        </is>
+      </c>
+      <c r="C1" s="14" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D1" s="14" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="E1" s="14" t="inlineStr">
+        <is>
+          <t>Power 0 — auto</t>
+        </is>
+      </c>
+      <c r="F1" s="14" t="inlineStr">
+        <is>
+          <t>Power 1</t>
+        </is>
+      </c>
+      <c r="G1" s="14" t="inlineStr">
+        <is>
+          <t>Power 2</t>
+        </is>
+      </c>
+      <c r="H1" s="14" t="inlineStr">
+        <is>
+          <t>Power 3</t>
+        </is>
+      </c>
+      <c r="I1" s="14" t="inlineStr">
+        <is>
+          <t>Power 4</t>
+        </is>
+      </c>
+      <c r="J1" s="14" t="inlineStr">
+        <is>
+          <t>Power 5</t>
+        </is>
+      </c>
+      <c r="L1" s="15" t="inlineStr">
+        <is>
+          <t>HOW POWERS ARE SHARED</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Bramwen</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Earth</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+      <c r="E2" s="16" t="inlineStr">
+        <is>
+          <t>Sundered Ground</t>
+        </is>
+      </c>
+      <c r="F2" s="17" t="inlineStr">
+        <is>
+          <t>Root and Hold</t>
+        </is>
+      </c>
+      <c r="G2" s="17" t="inlineStr">
+        <is>
+          <t>The Mountain Answers</t>
+        </is>
+      </c>
+      <c r="H2" s="18" t="inlineStr">
+        <is>
+          <t>The Bloom Lends Heat</t>
+        </is>
+      </c>
+      <c r="I2" s="19" t="inlineStr">
+        <is>
+          <t>Years in the Making</t>
+        </is>
+      </c>
+      <c r="J2" s="19" t="inlineStr">
+        <is>
+          <t>Wrath of the Slow Stone</t>
+        </is>
+      </c>
+      <c r="L2" s="20" t="inlineStr">
+        <is>
+          <t>Power 0 — auto-skill. The default attack, usable every turn with</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Ossic</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Earth</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Dark</t>
+        </is>
+      </c>
+      <c r="E3" s="16" t="inlineStr">
+        <is>
+          <t>Sundered Ground</t>
+        </is>
+      </c>
+      <c r="F3" s="17" t="inlineStr">
+        <is>
+          <t>Root and Hold</t>
+        </is>
+      </c>
+      <c r="G3" s="17" t="inlineStr">
+        <is>
+          <t>The Mountain Answers</t>
+        </is>
+      </c>
+      <c r="H3" s="18" t="inlineStr">
+        <is>
+          <t>The Silence Lends Cover</t>
+        </is>
+      </c>
+      <c r="I3" s="19" t="inlineStr">
+        <is>
+          <t>Kneel and Raise</t>
+        </is>
+      </c>
+      <c r="J3" s="19" t="inlineStr">
+        <is>
+          <t>The God-Bone Wakes</t>
+        </is>
+      </c>
+      <c r="L3" s="20" t="inlineStr">
+        <is>
+          <t>no cooldown, so a hero is never idle. Shared by primary type.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Terragosa</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Earth</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="E4" s="16" t="inlineStr">
+        <is>
+          <t>Sundered Ground</t>
+        </is>
+      </c>
+      <c r="F4" s="17" t="inlineStr">
+        <is>
+          <t>Root and Hold</t>
+        </is>
+      </c>
+      <c r="G4" s="17" t="inlineStr">
+        <is>
+          <t>The Mountain Answers</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>The Word Lends Sight</t>
+        </is>
+      </c>
+      <c r="I4" s="19" t="inlineStr">
+        <is>
+          <t>Orchard Over Ruin</t>
+        </is>
+      </c>
+      <c r="J4" s="19" t="inlineStr">
+        <is>
+          <t>The Green Crown Descends</t>
+        </is>
+      </c>
+      <c r="L4" s="20" t="inlineStr">
+        <is>
+          <t>Powers 1-2 — shared by every hero of the same PRIMARY type.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Zephyrine</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Air</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="E5" s="16" t="inlineStr">
+        <is>
+          <t>Cutting Gale</t>
+        </is>
+      </c>
+      <c r="F5" s="17" t="inlineStr">
+        <is>
+          <t>Thin the Air</t>
+        </is>
+      </c>
+      <c r="G5" s="17" t="inlineStr">
+        <is>
+          <t>The Sky Unmoored</t>
+        </is>
+      </c>
+      <c r="H5" s="18" t="inlineStr">
+        <is>
+          <t>The Word Lends Sight</t>
+        </is>
+      </c>
+      <c r="I5" s="19" t="inlineStr">
+        <is>
+          <t>A Distance Never Closed</t>
+        </is>
+      </c>
+      <c r="J5" s="19" t="inlineStr">
+        <is>
+          <t>The Thin Blade Falls</t>
+        </is>
+      </c>
+      <c r="L5" s="20" t="inlineStr">
+        <is>
+          <t>9 types x 3 = 27 names. Three champions of a House share them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Cirrolan</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Air</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="E6" s="16" t="inlineStr">
+        <is>
+          <t>Cutting Gale</t>
+        </is>
+      </c>
+      <c r="F6" s="17" t="inlineStr">
+        <is>
+          <t>Thin the Air</t>
+        </is>
+      </c>
+      <c r="G6" s="17" t="inlineStr">
+        <is>
+          <t>The Sky Unmoored</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>The Tide Lends Patience</t>
+        </is>
+      </c>
+      <c r="I6" s="19" t="inlineStr">
+        <is>
+          <t>Rumour and Storm</t>
+        </is>
+      </c>
+      <c r="J6" s="19" t="inlineStr">
+        <is>
+          <t>Whisper from the High Reach</t>
+        </is>
+      </c>
+      <c r="L6" s="20" t="inlineStr">
+        <is>
+          <t>Power 3 — shared by every hero of the same SECONDARY type.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Vael</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Air</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Dark</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>Cutting Gale</t>
+        </is>
+      </c>
+      <c r="F7" s="17" t="inlineStr">
+        <is>
+          <t>Thin the Air</t>
+        </is>
+      </c>
+      <c r="G7" s="17" t="inlineStr">
+        <is>
+          <t>The Sky Unmoored</t>
+        </is>
+      </c>
+      <c r="H7" s="18" t="inlineStr">
+        <is>
+          <t>The Silence Lends Cover</t>
+        </is>
+      </c>
+      <c r="I7" s="19" t="inlineStr">
+        <is>
+          <t>Jump First</t>
+        </is>
+      </c>
+      <c r="J7" s="19" t="inlineStr">
+        <is>
+          <t>Nothing to Catch You</t>
+        </is>
+      </c>
+      <c r="L7" s="20" t="inlineStr">
+        <is>
+          <t>Only 6 names: melee always takes an arcane secondary, so no</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Ember Saelith</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Air</t>
+        </is>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>Ember Lash</t>
+        </is>
+      </c>
+      <c r="F8" s="17" t="inlineStr">
+        <is>
+          <t>Feed the Bloom</t>
+        </is>
+      </c>
+      <c r="G8" s="17" t="inlineStr">
+        <is>
+          <t>Everything Burns Twice</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>The Sky Lends Swiftness</t>
+        </is>
+      </c>
+      <c r="I8" s="19" t="inlineStr">
+        <is>
+          <t>The Room Warms</t>
+        </is>
+      </c>
+      <c r="J8" s="19" t="inlineStr">
+        <is>
+          <t>First Spark, Last Laugh</t>
+        </is>
+      </c>
+      <c r="L8" s="20" t="inlineStr">
+        <is>
+          <t>melee type ever appears here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Pyrrhic</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="E9" s="16" t="inlineStr">
+        <is>
+          <t>Ember Lash</t>
+        </is>
+      </c>
+      <c r="F9" s="17" t="inlineStr">
+        <is>
+          <t>Feed the Bloom</t>
+        </is>
+      </c>
+      <c r="G9" s="17" t="inlineStr">
+        <is>
+          <t>Everything Burns Twice</t>
+        </is>
+      </c>
+      <c r="H9" s="18" t="inlineStr">
+        <is>
+          <t>The Word Lends Sight</t>
+        </is>
+      </c>
+      <c r="I9" s="19" t="inlineStr">
+        <is>
+          <t>Less Left to Lose</t>
+        </is>
+      </c>
+      <c r="J9" s="19" t="inlineStr">
+        <is>
+          <t>Glad Ruin</t>
+        </is>
+      </c>
+      <c r="L9" s="20" t="inlineStr">
+        <is>
+          <t>Powers 4-5 — unique to the hero. 54 names, the identity layer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Cindara</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Earth</t>
+        </is>
+      </c>
+      <c r="E10" s="16" t="inlineStr">
+        <is>
+          <t>Ember Lash</t>
+        </is>
+      </c>
+      <c r="F10" s="17" t="inlineStr">
+        <is>
+          <t>Feed the Bloom</t>
+        </is>
+      </c>
+      <c r="G10" s="17" t="inlineStr">
+        <is>
+          <t>Everything Burns Twice</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>The Deep Lends Weight</t>
+        </is>
+      </c>
+      <c r="I10" s="19" t="inlineStr">
+        <is>
+          <t>The Coal, Not the Flame</t>
+        </is>
+      </c>
+      <c r="J10" s="19" t="inlineStr">
+        <is>
+          <t>The Long Burn</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Marisel</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Dark</t>
+        </is>
+      </c>
+      <c r="E11" s="16" t="inlineStr">
+        <is>
+          <t>Undertow</t>
+        </is>
+      </c>
+      <c r="F11" s="17" t="inlineStr">
+        <is>
+          <t>Wear the Stone</t>
+        </is>
+      </c>
+      <c r="G11" s="17" t="inlineStr">
+        <is>
+          <t>The Tide Remembers</t>
+        </is>
+      </c>
+      <c r="H11" s="18" t="inlineStr">
+        <is>
+          <t>The Silence Lends Cover</t>
+        </is>
+      </c>
+      <c r="I11" s="19" t="inlineStr">
+        <is>
+          <t>Your Own Past, Rising</t>
+        </is>
+      </c>
+      <c r="J11" s="19" t="inlineStr">
+        <is>
+          <t>Drown in What You Did</t>
+        </is>
+      </c>
+      <c r="L11" s="20" t="inlineStr">
+        <is>
+          <t>Names only. Effects, costs and cooldowns are not designed yet —</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Tidewarden Coll</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Earth</t>
+        </is>
+      </c>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>Undertow</t>
+        </is>
+      </c>
+      <c r="F12" s="17" t="inlineStr">
+        <is>
+          <t>Wear the Stone</t>
+        </is>
+      </c>
+      <c r="G12" s="17" t="inlineStr">
+        <is>
+          <t>The Tide Remembers</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>The Deep Lends Weight</t>
+        </is>
+      </c>
+      <c r="I12" s="19" t="inlineStr">
+        <is>
+          <t>Give Ground, Take Coast</t>
+        </is>
+      </c>
+      <c r="J12" s="19" t="inlineStr">
+        <is>
+          <t>The Bulwark Holds</t>
+        </is>
+      </c>
+      <c r="L12" s="20" t="inlineStr">
+        <is>
+          <t>see mechanics/03-powers.md when it exists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Nix</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Air</t>
+        </is>
+      </c>
+      <c r="E13" s="16" t="inlineStr">
+        <is>
+          <t>Undertow</t>
+        </is>
+      </c>
+      <c r="F13" s="17" t="inlineStr">
+        <is>
+          <t>Wear the Stone</t>
+        </is>
+      </c>
+      <c r="G13" s="17" t="inlineStr">
+        <is>
+          <t>The Tide Remembers</t>
+        </is>
+      </c>
+      <c r="H13" s="18" t="inlineStr">
+        <is>
+          <t>The Sky Lends Swiftness</t>
+        </is>
+      </c>
+      <c r="I13" s="19" t="inlineStr">
+        <is>
+          <t>Perfectly Calm</t>
+        </is>
+      </c>
+      <c r="J13" s="19" t="inlineStr">
+        <is>
+          <t>The Still Pool Closes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Seraphel</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+      <c r="E14" s="16" t="inlineStr">
+        <is>
+          <t>Verdict Light</t>
+        </is>
+      </c>
+      <c r="F14" s="17" t="inlineStr">
+        <is>
+          <t>Nothing Hidden</t>
+        </is>
+      </c>
+      <c r="G14" s="17" t="inlineStr">
+        <is>
+          <t>The First Word Spoken</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>The Bloom Lends Heat</t>
+        </is>
+      </c>
+      <c r="I14" s="19" t="inlineStr">
+        <is>
+          <t>The Gaze Accuses</t>
+        </is>
+      </c>
+      <c r="J14" s="19" t="inlineStr">
+        <is>
+          <t>Sentence Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Lucen</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Air</t>
+        </is>
+      </c>
+      <c r="E15" s="16" t="inlineStr">
+        <is>
+          <t>Verdict Light</t>
+        </is>
+      </c>
+      <c r="F15" s="17" t="inlineStr">
+        <is>
+          <t>Nothing Hidden</t>
+        </is>
+      </c>
+      <c r="G15" s="17" t="inlineStr">
+        <is>
+          <t>The First Word Spoken</t>
+        </is>
+      </c>
+      <c r="H15" s="18" t="inlineStr">
+        <is>
+          <t>The Sky Lends Swiftness</t>
+        </is>
+      </c>
+      <c r="I15" s="19" t="inlineStr">
+        <is>
+          <t>Three Beams, No Shadow</t>
+        </is>
+      </c>
+      <c r="J15" s="19" t="inlineStr">
+        <is>
+          <t>The Unhidden Hour</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Auriel Dawnkeep</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="E16" s="16" t="inlineStr">
+        <is>
+          <t>Verdict Light</t>
+        </is>
+      </c>
+      <c r="F16" s="17" t="inlineStr">
+        <is>
+          <t>Nothing Hidden</t>
+        </is>
+      </c>
+      <c r="G16" s="17" t="inlineStr">
+        <is>
+          <t>The First Word Spoken</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>The Tide Lends Patience</t>
+        </is>
+      </c>
+      <c r="I16" s="19" t="inlineStr">
+        <is>
+          <t>The Lantern Holds</t>
+        </is>
+      </c>
+      <c r="J16" s="19" t="inlineStr">
+        <is>
+          <t>Last Light on the Wall</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Nyxara</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Dark</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="E17" s="16" t="inlineStr">
+        <is>
+          <t>Veilcut</t>
+        </is>
+      </c>
+      <c r="F17" s="17" t="inlineStr">
+        <is>
+          <t>Draw the Veil</t>
+        </is>
+      </c>
+      <c r="G17" s="17" t="inlineStr">
+        <is>
+          <t>The Last Silence</t>
+        </is>
+      </c>
+      <c r="H17" s="18" t="inlineStr">
+        <is>
+          <t>The Tide Lends Patience</t>
+        </is>
+      </c>
+      <c r="I17" s="19" t="inlineStr">
+        <is>
+          <t>A Kindness, Ending</t>
+        </is>
+      </c>
+      <c r="J17" s="19" t="inlineStr">
+        <is>
+          <t>Mercy at the End</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Umbriel</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Dark</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+      <c r="E18" s="16" t="inlineStr">
+        <is>
+          <t>Veilcut</t>
+        </is>
+      </c>
+      <c r="F18" s="17" t="inlineStr">
+        <is>
+          <t>Draw the Veil</t>
+        </is>
+      </c>
+      <c r="G18" s="17" t="inlineStr">
+        <is>
+          <t>The Last Silence</t>
+        </is>
+      </c>
+      <c r="H18" s="18" t="inlineStr">
+        <is>
+          <t>The Bloom Lends Heat</t>
+        </is>
+      </c>
+      <c r="I18" s="19" t="inlineStr">
+        <is>
+          <t>Unwrite the Line</t>
+        </is>
+      </c>
+      <c r="J18" s="19" t="inlineStr">
+        <is>
+          <t>The Undoing</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Corvane</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Dark</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Earth</t>
+        </is>
+      </c>
+      <c r="E19" s="16" t="inlineStr">
+        <is>
+          <t>Veilcut</t>
+        </is>
+      </c>
+      <c r="F19" s="17" t="inlineStr">
+        <is>
+          <t>Draw the Veil</t>
+        </is>
+      </c>
+      <c r="G19" s="17" t="inlineStr">
+        <is>
+          <t>The Last Silence</t>
+        </is>
+      </c>
+      <c r="H19" s="18" t="inlineStr">
+        <is>
+          <t>The Deep Lends Weight</t>
+        </is>
+      </c>
+      <c r="I19" s="19" t="inlineStr">
+        <is>
+          <t>I Know Your Hour</t>
+        </is>
+      </c>
+      <c r="J19" s="19" t="inlineStr">
+        <is>
+          <t>Shepherd of Endings</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Kaellis</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Slash</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="E20" s="16" t="inlineStr">
+        <is>
+          <t>Open Line</t>
+        </is>
+      </c>
+      <c r="F20" s="17" t="inlineStr">
+        <is>
+          <t>Riposte</t>
+        </is>
+      </c>
+      <c r="G20" s="17" t="inlineStr">
+        <is>
+          <t>One Clean Stroke</t>
+        </is>
+      </c>
+      <c r="H20" s="18" t="inlineStr">
+        <is>
+          <t>The Word Lends Sight</t>
+        </is>
+      </c>
+      <c r="I20" s="19" t="inlineStr">
+        <is>
+          <t>Never Twice</t>
+        </is>
+      </c>
+      <c r="J20" s="19" t="inlineStr">
+        <is>
+          <t>Immaculate</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Reyna Two-Rivers</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Slash</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="E21" s="16" t="inlineStr">
+        <is>
+          <t>Open Line</t>
+        </is>
+      </c>
+      <c r="F21" s="17" t="inlineStr">
+        <is>
+          <t>Riposte</t>
+        </is>
+      </c>
+      <c r="G21" s="17" t="inlineStr">
+        <is>
+          <t>One Clean Stroke</t>
+        </is>
+      </c>
+      <c r="H21" s="18" t="inlineStr">
+        <is>
+          <t>The Tide Lends Patience</t>
+        </is>
+      </c>
+      <c r="I21" s="19" t="inlineStr">
+        <is>
+          <t>Two Rivers Meeting</t>
+        </is>
+      </c>
+      <c r="J21" s="19" t="inlineStr">
+        <is>
+          <t>The Current Takes All</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Grieve</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Slash</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Dark</t>
+        </is>
+      </c>
+      <c r="E22" s="16" t="inlineStr">
+        <is>
+          <t>Open Line</t>
+        </is>
+      </c>
+      <c r="F22" s="17" t="inlineStr">
+        <is>
+          <t>Riposte</t>
+        </is>
+      </c>
+      <c r="G22" s="17" t="inlineStr">
+        <is>
+          <t>One Clean Stroke</t>
+        </is>
+      </c>
+      <c r="H22" s="18" t="inlineStr">
+        <is>
+          <t>The Silence Lends Cover</t>
+        </is>
+      </c>
+      <c r="I22" s="19" t="inlineStr">
+        <is>
+          <t>Clear the Room</t>
+        </is>
+      </c>
+      <c r="J22" s="19" t="inlineStr">
+        <is>
+          <t>The Wide Reaping</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Vantric</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Pierce</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Air</t>
+        </is>
+      </c>
+      <c r="E23" s="16" t="inlineStr">
+        <is>
+          <t>Seamfinder</t>
+        </is>
+      </c>
+      <c r="F23" s="17" t="inlineStr">
+        <is>
+          <t>Thread the Guard</t>
+        </is>
+      </c>
+      <c r="G23" s="17" t="inlineStr">
+        <is>
+          <t>The Single Truth</t>
+        </is>
+      </c>
+      <c r="H23" s="18" t="inlineStr">
+        <is>
+          <t>The Sky Lends Swiftness</t>
+        </is>
+      </c>
+      <c r="I23" s="19" t="inlineStr">
+        <is>
+          <t>The One Gap</t>
+        </is>
+      </c>
+      <c r="J23" s="19" t="inlineStr">
+        <is>
+          <t>The Spear Finds It</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Silka Pinquick</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Pierce</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Dark</t>
+        </is>
+      </c>
+      <c r="E24" s="16" t="inlineStr">
+        <is>
+          <t>Seamfinder</t>
+        </is>
+      </c>
+      <c r="F24" s="17" t="inlineStr">
+        <is>
+          <t>Thread the Guard</t>
+        </is>
+      </c>
+      <c r="G24" s="17" t="inlineStr">
+        <is>
+          <t>The Single Truth</t>
+        </is>
+      </c>
+      <c r="H24" s="18" t="inlineStr">
+        <is>
+          <t>The Silence Lends Cover</t>
+        </is>
+      </c>
+      <c r="I24" s="19" t="inlineStr">
+        <is>
+          <t>Already Behind You</t>
+        </is>
+      </c>
+      <c r="J24" s="19" t="inlineStr">
+        <is>
+          <t>Quicker Than Told</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Lord Aiguille</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Pierce</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="E25" s="16" t="inlineStr">
+        <is>
+          <t>Seamfinder</t>
+        </is>
+      </c>
+      <c r="F25" s="17" t="inlineStr">
+        <is>
+          <t>Thread the Guard</t>
+        </is>
+      </c>
+      <c r="G25" s="17" t="inlineStr">
+        <is>
+          <t>The Single Truth</t>
+        </is>
+      </c>
+      <c r="H25" s="18" t="inlineStr">
+        <is>
+          <t>The Word Lends Sight</t>
+        </is>
+      </c>
+      <c r="I25" s="19" t="inlineStr">
+        <is>
+          <t>Before You Decide</t>
+        </is>
+      </c>
+      <c r="J25" s="19" t="inlineStr">
+        <is>
+          <t>The Long Point</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Boldrek</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Crush</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="E26" s="16" t="inlineStr">
+        <is>
+          <t>Deadweight</t>
+        </is>
+      </c>
+      <c r="F26" s="17" t="inlineStr">
+        <is>
+          <t>Make an Opening</t>
+        </is>
+      </c>
+      <c r="G26" s="17" t="inlineStr">
+        <is>
+          <t>The Sky Falls</t>
+        </is>
+      </c>
+      <c r="H26" s="18" t="inlineStr">
+        <is>
+          <t>The Word Lends Sight</t>
+        </is>
+      </c>
+      <c r="I26" s="19" t="inlineStr">
+        <is>
+          <t>All At Once</t>
+        </is>
+      </c>
+      <c r="J26" s="19" t="inlineStr">
+        <is>
+          <t>Avalanche</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Hettamar Ironfall</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Crush</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Dark</t>
+        </is>
+      </c>
+      <c r="E27" s="16" t="inlineStr">
+        <is>
+          <t>Deadweight</t>
+        </is>
+      </c>
+      <c r="F27" s="17" t="inlineStr">
+        <is>
+          <t>Make an Opening</t>
+        </is>
+      </c>
+      <c r="G27" s="17" t="inlineStr">
+        <is>
+          <t>The Sky Falls</t>
+        </is>
+      </c>
+      <c r="H27" s="18" t="inlineStr">
+        <is>
+          <t>The Silence Lends Cover</t>
+        </is>
+      </c>
+      <c r="I27" s="19" t="inlineStr">
+        <is>
+          <t>End of Argument</t>
+        </is>
+      </c>
+      <c r="J27" s="19" t="inlineStr">
+        <is>
+          <t>Ironfall</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Mauless</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Crush</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Earth</t>
+        </is>
+      </c>
+      <c r="E28" s="16" t="inlineStr">
+        <is>
+          <t>Deadweight</t>
+        </is>
+      </c>
+      <c r="F28" s="17" t="inlineStr">
+        <is>
+          <t>Make an Opening</t>
+        </is>
+      </c>
+      <c r="G28" s="17" t="inlineStr">
+        <is>
+          <t>The Sky Falls</t>
+        </is>
+      </c>
+      <c r="H28" s="18" t="inlineStr">
+        <is>
+          <t>The Deep Lends Weight</t>
+        </is>
+      </c>
+      <c r="I28" s="19" t="inlineStr">
+        <is>
+          <t>Guards Break First</t>
+        </is>
+      </c>
+      <c r="J28" s="19" t="inlineStr">
+        <is>
+          <t>The Undenied</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J28"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add Role to the Powers grid and a distinct-power list sheet
Role moves into column B of Powers, shifting the rest right one — a
power has to read well for every hero that gets it, and role is the
strongest signal of that for the shared tiers.

Power List is one row per distinct name, 87 of them: the granting
type, every owning hero with its role, and a wide Prompt column for
what the power should do. Rerunning the generator carries authored
prompts across, matched on the power name.
</commit_message>
<xml_diff>
--- a/resources/characters/hero-stats.xlsx
+++ b/resources/characters/hero-stats.xlsx
@@ -5,11 +5,13 @@
   <sheets>
     <sheet name="Hero Stats" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Powers" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Rules" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Power List" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Rules" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hero Stats'!$A$1:$W$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Powers'!$A$1:$J$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Powers'!$A$1:$K$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Power List'!$A$1:$F$88</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -18,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -76,6 +78,9 @@
     </font>
     <font>
       <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="10">
@@ -141,7 +146,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -175,6 +180,16 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7004,20 +7019,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:M28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="13" min="1" max="1"/>
-    <col width="20" customWidth="1" style="13" min="2" max="2"/>
-    <col width="11" customWidth="1" style="13" min="3" max="3"/>
-    <col width="12" customWidth="1" style="13" min="4" max="4"/>
-    <col width="22" customWidth="1" style="13" min="5" max="5"/>
+    <col width="10" customWidth="1" style="13" min="2" max="2"/>
+    <col width="20" customWidth="1" style="13" min="3" max="3"/>
+    <col width="11" customWidth="1" style="13" min="4" max="4"/>
+    <col width="12" customWidth="1" style="13" min="5" max="5"/>
     <col width="22" customWidth="1" style="13" min="6" max="6"/>
-    <col width="26" customWidth="1" style="13" min="7" max="7"/>
+    <col width="22" customWidth="1" style="13" min="7" max="7"/>
     <col width="26" customWidth="1" style="13" min="8" max="8"/>
     <col width="26" customWidth="1" style="13" min="9" max="9"/>
-    <col width="28" customWidth="1" style="13" min="10" max="10"/>
-    <col width="66" customWidth="1" style="13" min="12" max="12"/>
+    <col width="26" customWidth="1" style="13" min="10" max="10"/>
+    <col width="28" customWidth="1" style="13" min="11" max="11"/>
+    <col width="66" customWidth="1" style="13" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="13">
@@ -7028,50 +7044,55 @@
       </c>
       <c r="B1" s="14" t="inlineStr">
         <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C1" s="14" t="inlineStr">
+        <is>
           <t>Hero</t>
         </is>
       </c>
-      <c r="C1" s="14" t="inlineStr">
+      <c r="D1" s="14" t="inlineStr">
         <is>
           <t>Primary</t>
         </is>
       </c>
-      <c r="D1" s="14" t="inlineStr">
+      <c r="E1" s="14" t="inlineStr">
         <is>
           <t>Secondary</t>
         </is>
       </c>
-      <c r="E1" s="14" t="inlineStr">
+      <c r="F1" s="14" t="inlineStr">
         <is>
           <t>Power 0 — auto</t>
         </is>
       </c>
-      <c r="F1" s="14" t="inlineStr">
+      <c r="G1" s="14" t="inlineStr">
         <is>
           <t>Power 1</t>
         </is>
       </c>
-      <c r="G1" s="14" t="inlineStr">
+      <c r="H1" s="14" t="inlineStr">
         <is>
           <t>Power 2</t>
         </is>
       </c>
-      <c r="H1" s="14" t="inlineStr">
+      <c r="I1" s="14" t="inlineStr">
         <is>
           <t>Power 3</t>
         </is>
       </c>
-      <c r="I1" s="14" t="inlineStr">
+      <c r="J1" s="14" t="inlineStr">
         <is>
           <t>Power 4</t>
         </is>
       </c>
-      <c r="J1" s="14" t="inlineStr">
+      <c r="K1" s="14" t="inlineStr">
         <is>
           <t>Power 5</t>
         </is>
       </c>
-      <c r="L1" s="15" t="inlineStr">
+      <c r="M1" s="15" t="inlineStr">
         <is>
           <t>HOW POWERS ARE SHARED</t>
         </is>
@@ -7083,50 +7104,55 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Striker</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>Bramwen</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Earth</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Fire</t>
         </is>
       </c>
-      <c r="E2" s="16" t="inlineStr">
+      <c r="F2" s="16" t="inlineStr">
         <is>
           <t>Sundered Ground</t>
         </is>
       </c>
-      <c r="F2" s="17" t="inlineStr">
+      <c r="G2" s="17" t="inlineStr">
         <is>
           <t>Root and Hold</t>
         </is>
       </c>
-      <c r="G2" s="17" t="inlineStr">
+      <c r="H2" s="17" t="inlineStr">
         <is>
           <t>The Mountain Answers</t>
         </is>
       </c>
-      <c r="H2" s="18" t="inlineStr">
+      <c r="I2" s="18" t="inlineStr">
         <is>
           <t>The Bloom Lends Heat</t>
         </is>
       </c>
-      <c r="I2" s="19" t="inlineStr">
+      <c r="J2" s="19" t="inlineStr">
         <is>
           <t>Years in the Making</t>
         </is>
       </c>
-      <c r="J2" s="19" t="inlineStr">
+      <c r="K2" s="19" t="inlineStr">
         <is>
           <t>Wrath of the Slow Stone</t>
         </is>
       </c>
-      <c r="L2" s="20" t="inlineStr">
+      <c r="M2" s="20" t="inlineStr">
         <is>
           <t>Power 0 — auto-skill. The default attack, usable every turn with</t>
         </is>
@@ -7138,50 +7164,55 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>Tank</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>Ossic</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Earth</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Dark</t>
         </is>
       </c>
-      <c r="E3" s="16" t="inlineStr">
+      <c r="F3" s="16" t="inlineStr">
         <is>
           <t>Sundered Ground</t>
         </is>
       </c>
-      <c r="F3" s="17" t="inlineStr">
+      <c r="G3" s="17" t="inlineStr">
         <is>
           <t>Root and Hold</t>
         </is>
       </c>
-      <c r="G3" s="17" t="inlineStr">
+      <c r="H3" s="17" t="inlineStr">
         <is>
           <t>The Mountain Answers</t>
         </is>
       </c>
-      <c r="H3" s="18" t="inlineStr">
+      <c r="I3" s="18" t="inlineStr">
         <is>
           <t>The Silence Lends Cover</t>
         </is>
       </c>
-      <c r="I3" s="19" t="inlineStr">
+      <c r="J3" s="19" t="inlineStr">
         <is>
           <t>Kneel and Raise</t>
         </is>
       </c>
-      <c r="J3" s="19" t="inlineStr">
+      <c r="K3" s="19" t="inlineStr">
         <is>
           <t>The God-Bone Wakes</t>
         </is>
       </c>
-      <c r="L3" s="20" t="inlineStr">
+      <c r="M3" s="20" t="inlineStr">
         <is>
           <t>no cooldown, so a hero is never idle. Shared by primary type.</t>
         </is>
@@ -7193,50 +7224,55 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>Tank</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>Terragosa</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Earth</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Light</t>
         </is>
       </c>
-      <c r="E4" s="16" t="inlineStr">
+      <c r="F4" s="16" t="inlineStr">
         <is>
           <t>Sundered Ground</t>
         </is>
       </c>
-      <c r="F4" s="17" t="inlineStr">
+      <c r="G4" s="17" t="inlineStr">
         <is>
           <t>Root and Hold</t>
         </is>
       </c>
-      <c r="G4" s="17" t="inlineStr">
+      <c r="H4" s="17" t="inlineStr">
         <is>
           <t>The Mountain Answers</t>
         </is>
       </c>
-      <c r="H4" s="18" t="inlineStr">
+      <c r="I4" s="18" t="inlineStr">
         <is>
           <t>The Word Lends Sight</t>
         </is>
       </c>
-      <c r="I4" s="19" t="inlineStr">
+      <c r="J4" s="19" t="inlineStr">
         <is>
           <t>Orchard Over Ruin</t>
         </is>
       </c>
-      <c r="J4" s="19" t="inlineStr">
+      <c r="K4" s="19" t="inlineStr">
         <is>
           <t>The Green Crown Descends</t>
         </is>
       </c>
-      <c r="L4" s="20" t="inlineStr">
+      <c r="M4" s="20" t="inlineStr">
         <is>
           <t>Powers 1-2 — shared by every hero of the same PRIMARY type.</t>
         </is>
@@ -7248,50 +7284,55 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>Striker</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>Zephyrine</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Air</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Light</t>
         </is>
       </c>
-      <c r="E5" s="16" t="inlineStr">
+      <c r="F5" s="16" t="inlineStr">
         <is>
           <t>Cutting Gale</t>
         </is>
       </c>
-      <c r="F5" s="17" t="inlineStr">
+      <c r="G5" s="17" t="inlineStr">
         <is>
           <t>Thin the Air</t>
         </is>
       </c>
-      <c r="G5" s="17" t="inlineStr">
+      <c r="H5" s="17" t="inlineStr">
         <is>
           <t>The Sky Unmoored</t>
         </is>
       </c>
-      <c r="H5" s="18" t="inlineStr">
+      <c r="I5" s="18" t="inlineStr">
         <is>
           <t>The Word Lends Sight</t>
         </is>
       </c>
-      <c r="I5" s="19" t="inlineStr">
+      <c r="J5" s="19" t="inlineStr">
         <is>
           <t>A Distance Never Closed</t>
         </is>
       </c>
-      <c r="J5" s="19" t="inlineStr">
+      <c r="K5" s="19" t="inlineStr">
         <is>
           <t>The Thin Blade Falls</t>
         </is>
       </c>
-      <c r="L5" s="20" t="inlineStr">
+      <c r="M5" s="20" t="inlineStr">
         <is>
           <t>9 types x 3 = 27 names. Three champions of a House share them.</t>
         </is>
@@ -7303,50 +7344,55 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>Buffer</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>Cirrolan</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Air</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Water</t>
         </is>
       </c>
-      <c r="E6" s="16" t="inlineStr">
+      <c r="F6" s="16" t="inlineStr">
         <is>
           <t>Cutting Gale</t>
         </is>
       </c>
-      <c r="F6" s="17" t="inlineStr">
+      <c r="G6" s="17" t="inlineStr">
         <is>
           <t>Thin the Air</t>
         </is>
       </c>
-      <c r="G6" s="17" t="inlineStr">
+      <c r="H6" s="17" t="inlineStr">
         <is>
           <t>The Sky Unmoored</t>
         </is>
       </c>
-      <c r="H6" s="18" t="inlineStr">
+      <c r="I6" s="18" t="inlineStr">
         <is>
           <t>The Tide Lends Patience</t>
         </is>
       </c>
-      <c r="I6" s="19" t="inlineStr">
+      <c r="J6" s="19" t="inlineStr">
         <is>
           <t>Rumour and Storm</t>
         </is>
       </c>
-      <c r="J6" s="19" t="inlineStr">
+      <c r="K6" s="19" t="inlineStr">
         <is>
           <t>Whisper from the High Reach</t>
         </is>
       </c>
-      <c r="L6" s="20" t="inlineStr">
+      <c r="M6" s="20" t="inlineStr">
         <is>
           <t>Power 3 — shared by every hero of the same SECONDARY type.</t>
         </is>
@@ -7358,50 +7404,55 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>Ranged</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>Vael</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Air</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Dark</t>
         </is>
       </c>
-      <c r="E7" s="16" t="inlineStr">
+      <c r="F7" s="16" t="inlineStr">
         <is>
           <t>Cutting Gale</t>
         </is>
       </c>
-      <c r="F7" s="17" t="inlineStr">
+      <c r="G7" s="17" t="inlineStr">
         <is>
           <t>Thin the Air</t>
         </is>
       </c>
-      <c r="G7" s="17" t="inlineStr">
+      <c r="H7" s="17" t="inlineStr">
         <is>
           <t>The Sky Unmoored</t>
         </is>
       </c>
-      <c r="H7" s="18" t="inlineStr">
+      <c r="I7" s="18" t="inlineStr">
         <is>
           <t>The Silence Lends Cover</t>
         </is>
       </c>
-      <c r="I7" s="19" t="inlineStr">
+      <c r="J7" s="19" t="inlineStr">
         <is>
           <t>Jump First</t>
         </is>
       </c>
-      <c r="J7" s="19" t="inlineStr">
+      <c r="K7" s="19" t="inlineStr">
         <is>
           <t>Nothing to Catch You</t>
         </is>
       </c>
-      <c r="L7" s="20" t="inlineStr">
+      <c r="M7" s="20" t="inlineStr">
         <is>
           <t>Only 6 names: melee always takes an arcane secondary, so no</t>
         </is>
@@ -7413,50 +7464,55 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>Striker</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>Ember Saelith</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Fire</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>Air</t>
         </is>
       </c>
-      <c r="E8" s="16" t="inlineStr">
+      <c r="F8" s="16" t="inlineStr">
         <is>
           <t>Ember Lash</t>
         </is>
       </c>
-      <c r="F8" s="17" t="inlineStr">
+      <c r="G8" s="17" t="inlineStr">
         <is>
           <t>Feed the Bloom</t>
         </is>
       </c>
-      <c r="G8" s="17" t="inlineStr">
+      <c r="H8" s="17" t="inlineStr">
         <is>
           <t>Everything Burns Twice</t>
         </is>
       </c>
-      <c r="H8" s="18" t="inlineStr">
+      <c r="I8" s="18" t="inlineStr">
         <is>
           <t>The Sky Lends Swiftness</t>
         </is>
       </c>
-      <c r="I8" s="19" t="inlineStr">
+      <c r="J8" s="19" t="inlineStr">
         <is>
           <t>The Room Warms</t>
         </is>
       </c>
-      <c r="J8" s="19" t="inlineStr">
+      <c r="K8" s="19" t="inlineStr">
         <is>
           <t>First Spark, Last Laugh</t>
         </is>
       </c>
-      <c r="L8" s="20" t="inlineStr">
+      <c r="M8" s="20" t="inlineStr">
         <is>
           <t>melee type ever appears here.</t>
         </is>
@@ -7468,50 +7524,55 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>Ranged</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>Pyrrhic</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Fire</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>Light</t>
         </is>
       </c>
-      <c r="E9" s="16" t="inlineStr">
+      <c r="F9" s="16" t="inlineStr">
         <is>
           <t>Ember Lash</t>
         </is>
       </c>
-      <c r="F9" s="17" t="inlineStr">
+      <c r="G9" s="17" t="inlineStr">
         <is>
           <t>Feed the Bloom</t>
         </is>
       </c>
-      <c r="G9" s="17" t="inlineStr">
+      <c r="H9" s="17" t="inlineStr">
         <is>
           <t>Everything Burns Twice</t>
         </is>
       </c>
-      <c r="H9" s="18" t="inlineStr">
+      <c r="I9" s="18" t="inlineStr">
         <is>
           <t>The Word Lends Sight</t>
         </is>
       </c>
-      <c r="I9" s="19" t="inlineStr">
+      <c r="J9" s="19" t="inlineStr">
         <is>
           <t>Less Left to Lose</t>
         </is>
       </c>
-      <c r="J9" s="19" t="inlineStr">
+      <c r="K9" s="19" t="inlineStr">
         <is>
           <t>Glad Ruin</t>
         </is>
       </c>
-      <c r="L9" s="20" t="inlineStr">
+      <c r="M9" s="20" t="inlineStr">
         <is>
           <t>Powers 4-5 — unique to the hero. 54 names, the identity layer.</t>
         </is>
@@ -7523,49 +7584,55 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>Ranged</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>Cindara</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Fire</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>Earth</t>
         </is>
       </c>
-      <c r="E10" s="16" t="inlineStr">
+      <c r="F10" s="16" t="inlineStr">
         <is>
           <t>Ember Lash</t>
         </is>
       </c>
-      <c r="F10" s="17" t="inlineStr">
+      <c r="G10" s="17" t="inlineStr">
         <is>
           <t>Feed the Bloom</t>
         </is>
       </c>
-      <c r="G10" s="17" t="inlineStr">
+      <c r="H10" s="17" t="inlineStr">
         <is>
           <t>Everything Burns Twice</t>
         </is>
       </c>
-      <c r="H10" s="18" t="inlineStr">
+      <c r="I10" s="18" t="inlineStr">
         <is>
           <t>The Deep Lends Weight</t>
         </is>
       </c>
-      <c r="I10" s="19" t="inlineStr">
+      <c r="J10" s="19" t="inlineStr">
         <is>
           <t>The Coal, Not the Flame</t>
         </is>
       </c>
-      <c r="J10" s="19" t="inlineStr">
+      <c r="K10" s="19" t="inlineStr">
         <is>
           <t>The Long Burn</t>
         </is>
       </c>
+      <c r="M10" s="20" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -7573,52 +7640,57 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>Striker</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
           <t>Marisel</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>Water</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>Dark</t>
         </is>
       </c>
-      <c r="E11" s="16" t="inlineStr">
+      <c r="F11" s="16" t="inlineStr">
         <is>
           <t>Undertow</t>
         </is>
       </c>
-      <c r="F11" s="17" t="inlineStr">
+      <c r="G11" s="17" t="inlineStr">
         <is>
           <t>Wear the Stone</t>
         </is>
       </c>
-      <c r="G11" s="17" t="inlineStr">
+      <c r="H11" s="17" t="inlineStr">
         <is>
           <t>The Tide Remembers</t>
         </is>
       </c>
-      <c r="H11" s="18" t="inlineStr">
+      <c r="I11" s="18" t="inlineStr">
         <is>
           <t>The Silence Lends Cover</t>
         </is>
       </c>
-      <c r="I11" s="19" t="inlineStr">
+      <c r="J11" s="19" t="inlineStr">
         <is>
           <t>Your Own Past, Rising</t>
         </is>
       </c>
-      <c r="J11" s="19" t="inlineStr">
+      <c r="K11" s="19" t="inlineStr">
         <is>
           <t>Drown in What You Did</t>
         </is>
       </c>
-      <c r="L11" s="20" t="inlineStr">
-        <is>
-          <t>Names only. Effects, costs and cooldowns are not designed yet —</t>
+      <c r="M11" s="20" t="inlineStr">
+        <is>
+          <t>Effects, costs and cooldowns are drafted on the Power List sheet —</t>
         </is>
       </c>
     </row>
@@ -7628,50 +7700,55 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>Ranged</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
           <t>Tidewarden Coll</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Water</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Earth</t>
         </is>
       </c>
-      <c r="E12" s="16" t="inlineStr">
+      <c r="F12" s="16" t="inlineStr">
         <is>
           <t>Undertow</t>
         </is>
       </c>
-      <c r="F12" s="17" t="inlineStr">
+      <c r="G12" s="17" t="inlineStr">
         <is>
           <t>Wear the Stone</t>
         </is>
       </c>
-      <c r="G12" s="17" t="inlineStr">
+      <c r="H12" s="17" t="inlineStr">
         <is>
           <t>The Tide Remembers</t>
         </is>
       </c>
-      <c r="H12" s="18" t="inlineStr">
+      <c r="I12" s="18" t="inlineStr">
         <is>
           <t>The Deep Lends Weight</t>
         </is>
       </c>
-      <c r="I12" s="19" t="inlineStr">
+      <c r="J12" s="19" t="inlineStr">
         <is>
           <t>Give Ground, Take Coast</t>
         </is>
       </c>
-      <c r="J12" s="19" t="inlineStr">
+      <c r="K12" s="19" t="inlineStr">
         <is>
           <t>The Bulwark Holds</t>
         </is>
       </c>
-      <c r="L12" s="20" t="inlineStr">
+      <c r="M12" s="20" t="inlineStr">
         <is>
           <t>see mechanics/03-powers.md when it exists.</t>
         </is>
@@ -7683,45 +7760,50 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>Ranged</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
           <t>Nix</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>Water</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>Air</t>
         </is>
       </c>
-      <c r="E13" s="16" t="inlineStr">
+      <c r="F13" s="16" t="inlineStr">
         <is>
           <t>Undertow</t>
         </is>
       </c>
-      <c r="F13" s="17" t="inlineStr">
+      <c r="G13" s="17" t="inlineStr">
         <is>
           <t>Wear the Stone</t>
         </is>
       </c>
-      <c r="G13" s="17" t="inlineStr">
+      <c r="H13" s="17" t="inlineStr">
         <is>
           <t>The Tide Remembers</t>
         </is>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>The Sky Lends Swiftness</t>
         </is>
       </c>
-      <c r="I13" s="19" t="inlineStr">
+      <c r="J13" s="19" t="inlineStr">
         <is>
           <t>Perfectly Calm</t>
         </is>
       </c>
-      <c r="J13" s="19" t="inlineStr">
+      <c r="K13" s="19" t="inlineStr">
         <is>
           <t>The Still Pool Closes</t>
         </is>
@@ -7733,45 +7815,50 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>Striker</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
           <t>Seraphel</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Light</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>Fire</t>
         </is>
       </c>
-      <c r="E14" s="16" t="inlineStr">
+      <c r="F14" s="16" t="inlineStr">
         <is>
           <t>Verdict Light</t>
         </is>
       </c>
-      <c r="F14" s="17" t="inlineStr">
+      <c r="G14" s="17" t="inlineStr">
         <is>
           <t>Nothing Hidden</t>
         </is>
       </c>
-      <c r="G14" s="17" t="inlineStr">
+      <c r="H14" s="17" t="inlineStr">
         <is>
           <t>The First Word Spoken</t>
         </is>
       </c>
-      <c r="H14" s="18" t="inlineStr">
+      <c r="I14" s="18" t="inlineStr">
         <is>
           <t>The Bloom Lends Heat</t>
         </is>
       </c>
-      <c r="I14" s="19" t="inlineStr">
+      <c r="J14" s="19" t="inlineStr">
         <is>
           <t>The Gaze Accuses</t>
         </is>
       </c>
-      <c r="J14" s="19" t="inlineStr">
+      <c r="K14" s="19" t="inlineStr">
         <is>
           <t>Sentence Passed</t>
         </is>
@@ -7783,45 +7870,50 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>Buffer</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
           <t>Lucen</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>Light</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>Air</t>
         </is>
       </c>
-      <c r="E15" s="16" t="inlineStr">
+      <c r="F15" s="16" t="inlineStr">
         <is>
           <t>Verdict Light</t>
         </is>
       </c>
-      <c r="F15" s="17" t="inlineStr">
+      <c r="G15" s="17" t="inlineStr">
         <is>
           <t>Nothing Hidden</t>
         </is>
       </c>
-      <c r="G15" s="17" t="inlineStr">
+      <c r="H15" s="17" t="inlineStr">
         <is>
           <t>The First Word Spoken</t>
         </is>
       </c>
-      <c r="H15" s="18" t="inlineStr">
+      <c r="I15" s="18" t="inlineStr">
         <is>
           <t>The Sky Lends Swiftness</t>
         </is>
       </c>
-      <c r="I15" s="19" t="inlineStr">
+      <c r="J15" s="19" t="inlineStr">
         <is>
           <t>Three Beams, No Shadow</t>
         </is>
       </c>
-      <c r="J15" s="19" t="inlineStr">
+      <c r="K15" s="19" t="inlineStr">
         <is>
           <t>The Unhidden Hour</t>
         </is>
@@ -7833,45 +7925,50 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>Tank</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
           <t>Auriel Dawnkeep</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>Light</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>Water</t>
         </is>
       </c>
-      <c r="E16" s="16" t="inlineStr">
+      <c r="F16" s="16" t="inlineStr">
         <is>
           <t>Verdict Light</t>
         </is>
       </c>
-      <c r="F16" s="17" t="inlineStr">
+      <c r="G16" s="17" t="inlineStr">
         <is>
           <t>Nothing Hidden</t>
         </is>
       </c>
-      <c r="G16" s="17" t="inlineStr">
+      <c r="H16" s="17" t="inlineStr">
         <is>
           <t>The First Word Spoken</t>
         </is>
       </c>
-      <c r="H16" s="18" t="inlineStr">
+      <c r="I16" s="18" t="inlineStr">
         <is>
           <t>The Tide Lends Patience</t>
         </is>
       </c>
-      <c r="I16" s="19" t="inlineStr">
+      <c r="J16" s="19" t="inlineStr">
         <is>
           <t>The Lantern Holds</t>
         </is>
       </c>
-      <c r="J16" s="19" t="inlineStr">
+      <c r="K16" s="19" t="inlineStr">
         <is>
           <t>Last Light on the Wall</t>
         </is>
@@ -7883,45 +7980,50 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>Striker</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
           <t>Nyxara</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>Dark</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>Water</t>
         </is>
       </c>
-      <c r="E17" s="16" t="inlineStr">
+      <c r="F17" s="16" t="inlineStr">
         <is>
           <t>Veilcut</t>
         </is>
       </c>
-      <c r="F17" s="17" t="inlineStr">
+      <c r="G17" s="17" t="inlineStr">
         <is>
           <t>Draw the Veil</t>
         </is>
       </c>
-      <c r="G17" s="17" t="inlineStr">
+      <c r="H17" s="17" t="inlineStr">
         <is>
           <t>The Last Silence</t>
         </is>
       </c>
-      <c r="H17" s="18" t="inlineStr">
+      <c r="I17" s="18" t="inlineStr">
         <is>
           <t>The Tide Lends Patience</t>
         </is>
       </c>
-      <c r="I17" s="19" t="inlineStr">
+      <c r="J17" s="19" t="inlineStr">
         <is>
           <t>A Kindness, Ending</t>
         </is>
       </c>
-      <c r="J17" s="19" t="inlineStr">
+      <c r="K17" s="19" t="inlineStr">
         <is>
           <t>Mercy at the End</t>
         </is>
@@ -7933,45 +8035,50 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>Buffer</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
           <t>Umbriel</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>Dark</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>Fire</t>
         </is>
       </c>
-      <c r="E18" s="16" t="inlineStr">
+      <c r="F18" s="16" t="inlineStr">
         <is>
           <t>Veilcut</t>
         </is>
       </c>
-      <c r="F18" s="17" t="inlineStr">
+      <c r="G18" s="17" t="inlineStr">
         <is>
           <t>Draw the Veil</t>
         </is>
       </c>
-      <c r="G18" s="17" t="inlineStr">
+      <c r="H18" s="17" t="inlineStr">
         <is>
           <t>The Last Silence</t>
         </is>
       </c>
-      <c r="H18" s="18" t="inlineStr">
+      <c r="I18" s="18" t="inlineStr">
         <is>
           <t>The Bloom Lends Heat</t>
         </is>
       </c>
-      <c r="I18" s="19" t="inlineStr">
+      <c r="J18" s="19" t="inlineStr">
         <is>
           <t>Unwrite the Line</t>
         </is>
       </c>
-      <c r="J18" s="19" t="inlineStr">
+      <c r="K18" s="19" t="inlineStr">
         <is>
           <t>The Undoing</t>
         </is>
@@ -7983,45 +8090,50 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>Tank</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
           <t>Corvane</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>Dark</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>Earth</t>
         </is>
       </c>
-      <c r="E19" s="16" t="inlineStr">
+      <c r="F19" s="16" t="inlineStr">
         <is>
           <t>Veilcut</t>
         </is>
       </c>
-      <c r="F19" s="17" t="inlineStr">
+      <c r="G19" s="17" t="inlineStr">
         <is>
           <t>Draw the Veil</t>
         </is>
       </c>
-      <c r="G19" s="17" t="inlineStr">
+      <c r="H19" s="17" t="inlineStr">
         <is>
           <t>The Last Silence</t>
         </is>
       </c>
-      <c r="H19" s="18" t="inlineStr">
+      <c r="I19" s="18" t="inlineStr">
         <is>
           <t>The Deep Lends Weight</t>
         </is>
       </c>
-      <c r="I19" s="19" t="inlineStr">
+      <c r="J19" s="19" t="inlineStr">
         <is>
           <t>I Know Your Hour</t>
         </is>
       </c>
-      <c r="J19" s="19" t="inlineStr">
+      <c r="K19" s="19" t="inlineStr">
         <is>
           <t>Shepherd of Endings</t>
         </is>
@@ -8033,45 +8145,50 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>Striker</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
           <t>Kaellis</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Slash</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>Light</t>
         </is>
       </c>
-      <c r="E20" s="16" t="inlineStr">
+      <c r="F20" s="16" t="inlineStr">
         <is>
           <t>Open Line</t>
         </is>
       </c>
-      <c r="F20" s="17" t="inlineStr">
+      <c r="G20" s="17" t="inlineStr">
         <is>
           <t>Riposte</t>
         </is>
       </c>
-      <c r="G20" s="17" t="inlineStr">
+      <c r="H20" s="17" t="inlineStr">
         <is>
           <t>One Clean Stroke</t>
         </is>
       </c>
-      <c r="H20" s="18" t="inlineStr">
+      <c r="I20" s="18" t="inlineStr">
         <is>
           <t>The Word Lends Sight</t>
         </is>
       </c>
-      <c r="I20" s="19" t="inlineStr">
+      <c r="J20" s="19" t="inlineStr">
         <is>
           <t>Never Twice</t>
         </is>
       </c>
-      <c r="J20" s="19" t="inlineStr">
+      <c r="K20" s="19" t="inlineStr">
         <is>
           <t>Immaculate</t>
         </is>
@@ -8083,45 +8200,50 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>Striker</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
           <t>Reyna Two-Rivers</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>Slash</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>Water</t>
         </is>
       </c>
-      <c r="E21" s="16" t="inlineStr">
+      <c r="F21" s="16" t="inlineStr">
         <is>
           <t>Open Line</t>
         </is>
       </c>
-      <c r="F21" s="17" t="inlineStr">
+      <c r="G21" s="17" t="inlineStr">
         <is>
           <t>Riposte</t>
         </is>
       </c>
-      <c r="G21" s="17" t="inlineStr">
+      <c r="H21" s="17" t="inlineStr">
         <is>
           <t>One Clean Stroke</t>
         </is>
       </c>
-      <c r="H21" s="18" t="inlineStr">
+      <c r="I21" s="18" t="inlineStr">
         <is>
           <t>The Tide Lends Patience</t>
         </is>
       </c>
-      <c r="I21" s="19" t="inlineStr">
+      <c r="J21" s="19" t="inlineStr">
         <is>
           <t>Two Rivers Meeting</t>
         </is>
       </c>
-      <c r="J21" s="19" t="inlineStr">
+      <c r="K21" s="19" t="inlineStr">
         <is>
           <t>The Current Takes All</t>
         </is>
@@ -8133,45 +8255,50 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>Tank</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
           <t>Grieve</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>Slash</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>Dark</t>
         </is>
       </c>
-      <c r="E22" s="16" t="inlineStr">
+      <c r="F22" s="16" t="inlineStr">
         <is>
           <t>Open Line</t>
         </is>
       </c>
-      <c r="F22" s="17" t="inlineStr">
+      <c r="G22" s="17" t="inlineStr">
         <is>
           <t>Riposte</t>
         </is>
       </c>
-      <c r="G22" s="17" t="inlineStr">
+      <c r="H22" s="17" t="inlineStr">
         <is>
           <t>One Clean Stroke</t>
         </is>
       </c>
-      <c r="H22" s="18" t="inlineStr">
+      <c r="I22" s="18" t="inlineStr">
         <is>
           <t>The Silence Lends Cover</t>
         </is>
       </c>
-      <c r="I22" s="19" t="inlineStr">
+      <c r="J22" s="19" t="inlineStr">
         <is>
           <t>Clear the Room</t>
         </is>
       </c>
-      <c r="J22" s="19" t="inlineStr">
+      <c r="K22" s="19" t="inlineStr">
         <is>
           <t>The Wide Reaping</t>
         </is>
@@ -8183,45 +8310,50 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>Striker</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
           <t>Vantric</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>Pierce</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>Air</t>
         </is>
       </c>
-      <c r="E23" s="16" t="inlineStr">
+      <c r="F23" s="16" t="inlineStr">
         <is>
           <t>Seamfinder</t>
         </is>
       </c>
-      <c r="F23" s="17" t="inlineStr">
+      <c r="G23" s="17" t="inlineStr">
         <is>
           <t>Thread the Guard</t>
         </is>
       </c>
-      <c r="G23" s="17" t="inlineStr">
+      <c r="H23" s="17" t="inlineStr">
         <is>
           <t>The Single Truth</t>
         </is>
       </c>
-      <c r="H23" s="18" t="inlineStr">
+      <c r="I23" s="18" t="inlineStr">
         <is>
           <t>The Sky Lends Swiftness</t>
         </is>
       </c>
-      <c r="I23" s="19" t="inlineStr">
+      <c r="J23" s="19" t="inlineStr">
         <is>
           <t>The One Gap</t>
         </is>
       </c>
-      <c r="J23" s="19" t="inlineStr">
+      <c r="K23" s="19" t="inlineStr">
         <is>
           <t>The Spear Finds It</t>
         </is>
@@ -8233,45 +8365,50 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
+          <t>Striker</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
           <t>Silka Pinquick</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>Pierce</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>Dark</t>
         </is>
       </c>
-      <c r="E24" s="16" t="inlineStr">
+      <c r="F24" s="16" t="inlineStr">
         <is>
           <t>Seamfinder</t>
         </is>
       </c>
-      <c r="F24" s="17" t="inlineStr">
+      <c r="G24" s="17" t="inlineStr">
         <is>
           <t>Thread the Guard</t>
         </is>
       </c>
-      <c r="G24" s="17" t="inlineStr">
+      <c r="H24" s="17" t="inlineStr">
         <is>
           <t>The Single Truth</t>
         </is>
       </c>
-      <c r="H24" s="18" t="inlineStr">
+      <c r="I24" s="18" t="inlineStr">
         <is>
           <t>The Silence Lends Cover</t>
         </is>
       </c>
-      <c r="I24" s="19" t="inlineStr">
+      <c r="J24" s="19" t="inlineStr">
         <is>
           <t>Already Behind You</t>
         </is>
       </c>
-      <c r="J24" s="19" t="inlineStr">
+      <c r="K24" s="19" t="inlineStr">
         <is>
           <t>Quicker Than Told</t>
         </is>
@@ -8283,45 +8420,50 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>Tank</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
           <t>Lord Aiguille</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>Pierce</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>Light</t>
         </is>
       </c>
-      <c r="E25" s="16" t="inlineStr">
+      <c r="F25" s="16" t="inlineStr">
         <is>
           <t>Seamfinder</t>
         </is>
       </c>
-      <c r="F25" s="17" t="inlineStr">
+      <c r="G25" s="17" t="inlineStr">
         <is>
           <t>Thread the Guard</t>
         </is>
       </c>
-      <c r="G25" s="17" t="inlineStr">
+      <c r="H25" s="17" t="inlineStr">
         <is>
           <t>The Single Truth</t>
         </is>
       </c>
-      <c r="H25" s="18" t="inlineStr">
+      <c r="I25" s="18" t="inlineStr">
         <is>
           <t>The Word Lends Sight</t>
         </is>
       </c>
-      <c r="I25" s="19" t="inlineStr">
+      <c r="J25" s="19" t="inlineStr">
         <is>
           <t>Before You Decide</t>
         </is>
       </c>
-      <c r="J25" s="19" t="inlineStr">
+      <c r="K25" s="19" t="inlineStr">
         <is>
           <t>The Long Point</t>
         </is>
@@ -8333,45 +8475,50 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
+          <t>Striker</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
           <t>Boldrek</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>Crush</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>Light</t>
         </is>
       </c>
-      <c r="E26" s="16" t="inlineStr">
+      <c r="F26" s="16" t="inlineStr">
         <is>
           <t>Deadweight</t>
         </is>
       </c>
-      <c r="F26" s="17" t="inlineStr">
+      <c r="G26" s="17" t="inlineStr">
         <is>
           <t>Make an Opening</t>
         </is>
       </c>
-      <c r="G26" s="17" t="inlineStr">
+      <c r="H26" s="17" t="inlineStr">
         <is>
           <t>The Sky Falls</t>
         </is>
       </c>
-      <c r="H26" s="18" t="inlineStr">
+      <c r="I26" s="18" t="inlineStr">
         <is>
           <t>The Word Lends Sight</t>
         </is>
       </c>
-      <c r="I26" s="19" t="inlineStr">
+      <c r="J26" s="19" t="inlineStr">
         <is>
           <t>All At Once</t>
         </is>
       </c>
-      <c r="J26" s="19" t="inlineStr">
+      <c r="K26" s="19" t="inlineStr">
         <is>
           <t>Avalanche</t>
         </is>
@@ -8383,45 +8530,50 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
+          <t>Striker</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
           <t>Hettamar Ironfall</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>Crush</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>Dark</t>
         </is>
       </c>
-      <c r="E27" s="16" t="inlineStr">
+      <c r="F27" s="16" t="inlineStr">
         <is>
           <t>Deadweight</t>
         </is>
       </c>
-      <c r="F27" s="17" t="inlineStr">
+      <c r="G27" s="17" t="inlineStr">
         <is>
           <t>Make an Opening</t>
         </is>
       </c>
-      <c r="G27" s="17" t="inlineStr">
+      <c r="H27" s="17" t="inlineStr">
         <is>
           <t>The Sky Falls</t>
         </is>
       </c>
-      <c r="H27" s="18" t="inlineStr">
+      <c r="I27" s="18" t="inlineStr">
         <is>
           <t>The Silence Lends Cover</t>
         </is>
       </c>
-      <c r="I27" s="19" t="inlineStr">
+      <c r="J27" s="19" t="inlineStr">
         <is>
           <t>End of Argument</t>
         </is>
       </c>
-      <c r="J27" s="19" t="inlineStr">
+      <c r="K27" s="19" t="inlineStr">
         <is>
           <t>Ironfall</t>
         </is>
@@ -8433,57 +8585,2450 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
+          <t>Tank</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
           <t>Mauless</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>Crush</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>Earth</t>
         </is>
       </c>
-      <c r="E28" s="16" t="inlineStr">
+      <c r="F28" s="16" t="inlineStr">
         <is>
           <t>Deadweight</t>
         </is>
       </c>
-      <c r="F28" s="17" t="inlineStr">
+      <c r="G28" s="17" t="inlineStr">
         <is>
           <t>Make an Opening</t>
         </is>
       </c>
-      <c r="G28" s="17" t="inlineStr">
+      <c r="H28" s="17" t="inlineStr">
         <is>
           <t>The Sky Falls</t>
         </is>
       </c>
-      <c r="H28" s="18" t="inlineStr">
+      <c r="I28" s="18" t="inlineStr">
         <is>
           <t>The Deep Lends Weight</t>
         </is>
       </c>
-      <c r="I28" s="19" t="inlineStr">
+      <c r="J28" s="19" t="inlineStr">
         <is>
           <t>Guards Break First</t>
         </is>
       </c>
-      <c r="J28" s="19" t="inlineStr">
+      <c r="K28" s="19" t="inlineStr">
         <is>
           <t>The Undenied</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J28"/>
+  <autoFilter ref="A1:K28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H88"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" style="13" min="1" max="1"/>
+    <col width="9" customWidth="1" style="13" min="2" max="2"/>
+    <col width="11" customWidth="1" style="13" min="3" max="3"/>
+    <col width="18" customWidth="1" style="13" min="4" max="4"/>
+    <col width="46" customWidth="1" style="13" min="5" max="5"/>
+    <col width="90" customWidth="1" style="13" min="6" max="6"/>
+    <col width="66" customWidth="1" style="13" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1" s="13">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>Power</t>
+        </is>
+      </c>
+      <c r="B1" s="14" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="C1" s="14" t="inlineStr">
+        <is>
+          <t>Shared via</t>
+        </is>
+      </c>
+      <c r="D1" s="14" t="inlineStr">
+        <is>
+          <t>Elements</t>
+        </is>
+      </c>
+      <c r="E1" s="14" t="inlineStr">
+        <is>
+          <t>Heroes</t>
+        </is>
+      </c>
+      <c r="F1" s="14" t="inlineStr">
+        <is>
+          <t>Prompt — what does it do?</t>
+        </is>
+      </c>
+      <c r="H1" s="15" t="inlineStr">
+        <is>
+          <t>ONE ROW PER DISTINCT POWER</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="21" t="inlineStr">
+        <is>
+          <t>Sundered Ground</t>
+        </is>
+      </c>
+      <c r="B2" s="22" t="inlineStr">
+        <is>
+          <t>0 — auto</t>
+        </is>
+      </c>
+      <c r="C2" s="22" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Earth</t>
+        </is>
+      </c>
+      <c r="E2" s="23" t="inlineStr">
+        <is>
+          <t>Bramwen (Striker) · Ossic (Tank) · Terragosa (Tank)</t>
+        </is>
+      </c>
+      <c r="F2" s="23" t="n"/>
+      <c r="H2" s="20" t="inlineStr">
+        <is>
+          <t>87 names: 27 shared by primary type (tiers 0-2), 6 shared by</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="21" t="inlineStr">
+        <is>
+          <t>Cutting Gale</t>
+        </is>
+      </c>
+      <c r="B3" s="22" t="inlineStr">
+        <is>
+          <t>0 — auto</t>
+        </is>
+      </c>
+      <c r="C3" s="22" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Air</t>
+        </is>
+      </c>
+      <c r="E3" s="23" t="inlineStr">
+        <is>
+          <t>Zephyrine (Striker) · Cirrolan (Buffer) · Vael (Ranged)</t>
+        </is>
+      </c>
+      <c r="F3" s="23" t="n"/>
+      <c r="H3" s="20" t="inlineStr">
+        <is>
+          <t>secondary type (tier 3), 54 unique to a hero (tiers 4-5).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="21" t="inlineStr">
+        <is>
+          <t>Ember Lash</t>
+        </is>
+      </c>
+      <c r="B4" s="22" t="inlineStr">
+        <is>
+          <t>0 — auto</t>
+        </is>
+      </c>
+      <c r="C4" s="22" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+      <c r="E4" s="23" t="inlineStr">
+        <is>
+          <t>Ember Saelith (Striker) · Pyrrhic (Ranged) · Cindara (Ranged)</t>
+        </is>
+      </c>
+      <c r="F4" s="23" t="n"/>
+      <c r="H4" s="20" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>Undertow</t>
+        </is>
+      </c>
+      <c r="B5" s="22" t="inlineStr">
+        <is>
+          <t>0 — auto</t>
+        </is>
+      </c>
+      <c r="C5" s="22" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="E5" s="23" t="inlineStr">
+        <is>
+          <t>Marisel (Striker) · Tidewarden Coll (Ranged) · Nix (Ranged)</t>
+        </is>
+      </c>
+      <c r="F5" s="23" t="n"/>
+      <c r="H5" s="20" t="inlineStr">
+        <is>
+          <t>Elements — the type that grants the power. For a unique power</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>Verdict Light</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>0 — auto</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="E6" s="23" t="inlineStr">
+        <is>
+          <t>Seraphel (Striker) · Lucen (Buffer) · Auriel Dawnkeep (Tank)</t>
+        </is>
+      </c>
+      <c r="F6" s="23" t="n"/>
+      <c r="H6" s="20" t="inlineStr">
+        <is>
+          <t>that is the owner's primary and secondary both.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>Veilcut</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>0 — auto</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Dark</t>
+        </is>
+      </c>
+      <c r="E7" s="23" t="inlineStr">
+        <is>
+          <t>Nyxara (Striker) · Umbriel (Buffer) · Corvane (Tank)</t>
+        </is>
+      </c>
+      <c r="F7" s="23" t="n"/>
+      <c r="H7" s="20" t="inlineStr">
+        <is>
+          <t>Heroes — every hero that gets this power, with its role, since</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>Open Line</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>0 — auto</t>
+        </is>
+      </c>
+      <c r="C8" s="22" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Slash</t>
+        </is>
+      </c>
+      <c r="E8" s="23" t="inlineStr">
+        <is>
+          <t>Kaellis (Striker) · Reyna Two-Rivers (Striker) · Grieve (Tank)</t>
+        </is>
+      </c>
+      <c r="F8" s="23" t="n"/>
+      <c r="H8" s="20" t="inlineStr">
+        <is>
+          <t>a shared power has to read well for all of them at once.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>Seamfinder</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
+        <is>
+          <t>0 — auto</t>
+        </is>
+      </c>
+      <c r="C9" s="22" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Pierce</t>
+        </is>
+      </c>
+      <c r="E9" s="23" t="inlineStr">
+        <is>
+          <t>Vantric (Striker) · Silka Pinquick (Striker) · Lord Aiguille (Tank)</t>
+        </is>
+      </c>
+      <c r="F9" s="23" t="n"/>
+      <c r="H9" s="20" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>Deadweight</t>
+        </is>
+      </c>
+      <c r="B10" s="22" t="inlineStr">
+        <is>
+          <t>0 — auto</t>
+        </is>
+      </c>
+      <c r="C10" s="22" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Crush</t>
+        </is>
+      </c>
+      <c r="E10" s="23" t="inlineStr">
+        <is>
+          <t>Boldrek (Striker) · Hettamar Ironfall (Striker) · Mauless (Tank)</t>
+        </is>
+      </c>
+      <c r="F10" s="23" t="n"/>
+      <c r="H10" s="20" t="inlineStr">
+        <is>
+          <t>Prompt — free text: what the power should do. Prompts survive a</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="24" t="inlineStr">
+        <is>
+          <t>Root and Hold</t>
+        </is>
+      </c>
+      <c r="B11" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="22" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Earth</t>
+        </is>
+      </c>
+      <c r="E11" s="23" t="inlineStr">
+        <is>
+          <t>Bramwen (Striker) · Ossic (Tank) · Terragosa (Tank)</t>
+        </is>
+      </c>
+      <c r="F11" s="23" t="n"/>
+      <c r="H11" s="20" t="inlineStr">
+        <is>
+          <t>rerun of tools/add-powers-sheet.py, matched on the power name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="24" t="inlineStr">
+        <is>
+          <t>Thin the Air</t>
+        </is>
+      </c>
+      <c r="B12" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="22" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Air</t>
+        </is>
+      </c>
+      <c r="E12" s="23" t="inlineStr">
+        <is>
+          <t>Zephyrine (Striker) · Cirrolan (Buffer) · Vael (Ranged)</t>
+        </is>
+      </c>
+      <c r="F12" s="23" t="n"/>
+      <c r="H12" s="20" t="inlineStr">
+        <is>
+          <t>Rename a power and its prompt is orphaned, not moved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="24" t="inlineStr">
+        <is>
+          <t>Feed the Bloom</t>
+        </is>
+      </c>
+      <c r="B13" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="22" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+      <c r="E13" s="23" t="inlineStr">
+        <is>
+          <t>Ember Saelith (Striker) · Pyrrhic (Ranged) · Cindara (Ranged)</t>
+        </is>
+      </c>
+      <c r="F13" s="23" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="24" t="inlineStr">
+        <is>
+          <t>Wear the Stone</t>
+        </is>
+      </c>
+      <c r="B14" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="22" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="E14" s="23" t="inlineStr">
+        <is>
+          <t>Marisel (Striker) · Tidewarden Coll (Ranged) · Nix (Ranged)</t>
+        </is>
+      </c>
+      <c r="F14" s="23" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="24" t="inlineStr">
+        <is>
+          <t>Nothing Hidden</t>
+        </is>
+      </c>
+      <c r="B15" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="22" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="E15" s="23" t="inlineStr">
+        <is>
+          <t>Seraphel (Striker) · Lucen (Buffer) · Auriel Dawnkeep (Tank)</t>
+        </is>
+      </c>
+      <c r="F15" s="23" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="24" t="inlineStr">
+        <is>
+          <t>Draw the Veil</t>
+        </is>
+      </c>
+      <c r="B16" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="22" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Dark</t>
+        </is>
+      </c>
+      <c r="E16" s="23" t="inlineStr">
+        <is>
+          <t>Nyxara (Striker) · Umbriel (Buffer) · Corvane (Tank)</t>
+        </is>
+      </c>
+      <c r="F16" s="23" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="24" t="inlineStr">
+        <is>
+          <t>Riposte</t>
+        </is>
+      </c>
+      <c r="B17" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="22" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Slash</t>
+        </is>
+      </c>
+      <c r="E17" s="23" t="inlineStr">
+        <is>
+          <t>Kaellis (Striker) · Reyna Two-Rivers (Striker) · Grieve (Tank)</t>
+        </is>
+      </c>
+      <c r="F17" s="23" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="24" t="inlineStr">
+        <is>
+          <t>Thread the Guard</t>
+        </is>
+      </c>
+      <c r="B18" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="22" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Pierce</t>
+        </is>
+      </c>
+      <c r="E18" s="23" t="inlineStr">
+        <is>
+          <t>Vantric (Striker) · Silka Pinquick (Striker) · Lord Aiguille (Tank)</t>
+        </is>
+      </c>
+      <c r="F18" s="23" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="24" t="inlineStr">
+        <is>
+          <t>Make an Opening</t>
+        </is>
+      </c>
+      <c r="B19" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" s="22" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Crush</t>
+        </is>
+      </c>
+      <c r="E19" s="23" t="inlineStr">
+        <is>
+          <t>Boldrek (Striker) · Hettamar Ironfall (Striker) · Mauless (Tank)</t>
+        </is>
+      </c>
+      <c r="F19" s="23" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="24" t="inlineStr">
+        <is>
+          <t>The Mountain Answers</t>
+        </is>
+      </c>
+      <c r="B20" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" s="22" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Earth</t>
+        </is>
+      </c>
+      <c r="E20" s="23" t="inlineStr">
+        <is>
+          <t>Bramwen (Striker) · Ossic (Tank) · Terragosa (Tank)</t>
+        </is>
+      </c>
+      <c r="F20" s="23" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="24" t="inlineStr">
+        <is>
+          <t>The Sky Unmoored</t>
+        </is>
+      </c>
+      <c r="B21" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" s="22" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Air</t>
+        </is>
+      </c>
+      <c r="E21" s="23" t="inlineStr">
+        <is>
+          <t>Zephyrine (Striker) · Cirrolan (Buffer) · Vael (Ranged)</t>
+        </is>
+      </c>
+      <c r="F21" s="23" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="24" t="inlineStr">
+        <is>
+          <t>Everything Burns Twice</t>
+        </is>
+      </c>
+      <c r="B22" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="C22" s="22" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+      <c r="E22" s="23" t="inlineStr">
+        <is>
+          <t>Ember Saelith (Striker) · Pyrrhic (Ranged) · Cindara (Ranged)</t>
+        </is>
+      </c>
+      <c r="F22" s="23" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="24" t="inlineStr">
+        <is>
+          <t>The Tide Remembers</t>
+        </is>
+      </c>
+      <c r="B23" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="C23" s="22" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="E23" s="23" t="inlineStr">
+        <is>
+          <t>Marisel (Striker) · Tidewarden Coll (Ranged) · Nix (Ranged)</t>
+        </is>
+      </c>
+      <c r="F23" s="23" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="24" t="inlineStr">
+        <is>
+          <t>The First Word Spoken</t>
+        </is>
+      </c>
+      <c r="B24" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" s="22" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="E24" s="23" t="inlineStr">
+        <is>
+          <t>Seraphel (Striker) · Lucen (Buffer) · Auriel Dawnkeep (Tank)</t>
+        </is>
+      </c>
+      <c r="F24" s="23" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="24" t="inlineStr">
+        <is>
+          <t>The Last Silence</t>
+        </is>
+      </c>
+      <c r="B25" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="C25" s="22" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Dark</t>
+        </is>
+      </c>
+      <c r="E25" s="23" t="inlineStr">
+        <is>
+          <t>Nyxara (Striker) · Umbriel (Buffer) · Corvane (Tank)</t>
+        </is>
+      </c>
+      <c r="F25" s="23" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="24" t="inlineStr">
+        <is>
+          <t>One Clean Stroke</t>
+        </is>
+      </c>
+      <c r="B26" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="C26" s="22" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Slash</t>
+        </is>
+      </c>
+      <c r="E26" s="23" t="inlineStr">
+        <is>
+          <t>Kaellis (Striker) · Reyna Two-Rivers (Striker) · Grieve (Tank)</t>
+        </is>
+      </c>
+      <c r="F26" s="23" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="24" t="inlineStr">
+        <is>
+          <t>The Single Truth</t>
+        </is>
+      </c>
+      <c r="B27" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" s="22" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Pierce</t>
+        </is>
+      </c>
+      <c r="E27" s="23" t="inlineStr">
+        <is>
+          <t>Vantric (Striker) · Silka Pinquick (Striker) · Lord Aiguille (Tank)</t>
+        </is>
+      </c>
+      <c r="F27" s="23" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="24" t="inlineStr">
+        <is>
+          <t>The Sky Falls</t>
+        </is>
+      </c>
+      <c r="B28" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="C28" s="22" t="inlineStr">
+        <is>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Crush</t>
+        </is>
+      </c>
+      <c r="E28" s="23" t="inlineStr">
+        <is>
+          <t>Boldrek (Striker) · Hettamar Ironfall (Striker) · Mauless (Tank)</t>
+        </is>
+      </c>
+      <c r="F28" s="23" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="25" t="inlineStr">
+        <is>
+          <t>The Bloom Lends Heat</t>
+        </is>
+      </c>
+      <c r="B29" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="C29" s="22" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+      <c r="E29" s="23" t="inlineStr">
+        <is>
+          <t>Bramwen (Striker) · Seraphel (Striker) · Umbriel (Buffer)</t>
+        </is>
+      </c>
+      <c r="F29" s="23" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="25" t="inlineStr">
+        <is>
+          <t>The Silence Lends Cover</t>
+        </is>
+      </c>
+      <c r="B30" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="C30" s="22" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Dark</t>
+        </is>
+      </c>
+      <c r="E30" s="23" t="inlineStr">
+        <is>
+          <t>Ossic (Tank) · Vael (Ranged) · Marisel (Striker) · Grieve (Tank) · Silka Pinquick (Striker) · Hettamar Ironfall (Striker)</t>
+        </is>
+      </c>
+      <c r="F30" s="23" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="25" t="inlineStr">
+        <is>
+          <t>The Word Lends Sight</t>
+        </is>
+      </c>
+      <c r="B31" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="C31" s="22" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="E31" s="23" t="inlineStr">
+        <is>
+          <t>Terragosa (Tank) · Zephyrine (Striker) · Pyrrhic (Ranged) · Kaellis (Striker) · Lord Aiguille (Tank) · Boldrek (Striker)</t>
+        </is>
+      </c>
+      <c r="F31" s="23" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="25" t="inlineStr">
+        <is>
+          <t>The Tide Lends Patience</t>
+        </is>
+      </c>
+      <c r="B32" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="C32" s="22" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Water</t>
+        </is>
+      </c>
+      <c r="E32" s="23" t="inlineStr">
+        <is>
+          <t>Cirrolan (Buffer) · Auriel Dawnkeep (Tank) · Nyxara (Striker) · Reyna Two-Rivers (Striker)</t>
+        </is>
+      </c>
+      <c r="F32" s="23" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="25" t="inlineStr">
+        <is>
+          <t>The Sky Lends Swiftness</t>
+        </is>
+      </c>
+      <c r="B33" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="C33" s="22" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Air</t>
+        </is>
+      </c>
+      <c r="E33" s="23" t="inlineStr">
+        <is>
+          <t>Ember Saelith (Striker) · Nix (Ranged) · Lucen (Buffer) · Vantric (Striker)</t>
+        </is>
+      </c>
+      <c r="F33" s="23" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="25" t="inlineStr">
+        <is>
+          <t>The Deep Lends Weight</t>
+        </is>
+      </c>
+      <c r="B34" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="C34" s="22" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Earth</t>
+        </is>
+      </c>
+      <c r="E34" s="23" t="inlineStr">
+        <is>
+          <t>Cindara (Ranged) · Tidewarden Coll (Ranged) · Corvane (Tank) · Mauless (Tank)</t>
+        </is>
+      </c>
+      <c r="F34" s="23" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="26" t="inlineStr">
+        <is>
+          <t>Years in the Making</t>
+        </is>
+      </c>
+      <c r="B35" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C35" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Earth · Fire</t>
+        </is>
+      </c>
+      <c r="E35" s="23" t="inlineStr">
+        <is>
+          <t>Bramwen (Striker)</t>
+        </is>
+      </c>
+      <c r="F35" s="23" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="26" t="inlineStr">
+        <is>
+          <t>Kneel and Raise</t>
+        </is>
+      </c>
+      <c r="B36" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C36" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Earth · Dark</t>
+        </is>
+      </c>
+      <c r="E36" s="23" t="inlineStr">
+        <is>
+          <t>Ossic (Tank)</t>
+        </is>
+      </c>
+      <c r="F36" s="23" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="26" t="inlineStr">
+        <is>
+          <t>Orchard Over Ruin</t>
+        </is>
+      </c>
+      <c r="B37" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C37" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Earth · Light</t>
+        </is>
+      </c>
+      <c r="E37" s="23" t="inlineStr">
+        <is>
+          <t>Terragosa (Tank)</t>
+        </is>
+      </c>
+      <c r="F37" s="23" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="26" t="inlineStr">
+        <is>
+          <t>A Distance Never Closed</t>
+        </is>
+      </c>
+      <c r="B38" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C38" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Air · Light</t>
+        </is>
+      </c>
+      <c r="E38" s="23" t="inlineStr">
+        <is>
+          <t>Zephyrine (Striker)</t>
+        </is>
+      </c>
+      <c r="F38" s="23" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="26" t="inlineStr">
+        <is>
+          <t>Rumour and Storm</t>
+        </is>
+      </c>
+      <c r="B39" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C39" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Air · Water</t>
+        </is>
+      </c>
+      <c r="E39" s="23" t="inlineStr">
+        <is>
+          <t>Cirrolan (Buffer)</t>
+        </is>
+      </c>
+      <c r="F39" s="23" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="26" t="inlineStr">
+        <is>
+          <t>Jump First</t>
+        </is>
+      </c>
+      <c r="B40" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C40" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Air · Dark</t>
+        </is>
+      </c>
+      <c r="E40" s="23" t="inlineStr">
+        <is>
+          <t>Vael (Ranged)</t>
+        </is>
+      </c>
+      <c r="F40" s="23" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="26" t="inlineStr">
+        <is>
+          <t>The Room Warms</t>
+        </is>
+      </c>
+      <c r="B41" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C41" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Fire · Air</t>
+        </is>
+      </c>
+      <c r="E41" s="23" t="inlineStr">
+        <is>
+          <t>Ember Saelith (Striker)</t>
+        </is>
+      </c>
+      <c r="F41" s="23" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="26" t="inlineStr">
+        <is>
+          <t>Less Left to Lose</t>
+        </is>
+      </c>
+      <c r="B42" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C42" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Fire · Light</t>
+        </is>
+      </c>
+      <c r="E42" s="23" t="inlineStr">
+        <is>
+          <t>Pyrrhic (Ranged)</t>
+        </is>
+      </c>
+      <c r="F42" s="23" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="26" t="inlineStr">
+        <is>
+          <t>The Coal, Not the Flame</t>
+        </is>
+      </c>
+      <c r="B43" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C43" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Fire · Earth</t>
+        </is>
+      </c>
+      <c r="E43" s="23" t="inlineStr">
+        <is>
+          <t>Cindara (Ranged)</t>
+        </is>
+      </c>
+      <c r="F43" s="23" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="26" t="inlineStr">
+        <is>
+          <t>Your Own Past, Rising</t>
+        </is>
+      </c>
+      <c r="B44" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C44" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Water · Dark</t>
+        </is>
+      </c>
+      <c r="E44" s="23" t="inlineStr">
+        <is>
+          <t>Marisel (Striker)</t>
+        </is>
+      </c>
+      <c r="F44" s="23" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="26" t="inlineStr">
+        <is>
+          <t>Give Ground, Take Coast</t>
+        </is>
+      </c>
+      <c r="B45" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C45" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Water · Earth</t>
+        </is>
+      </c>
+      <c r="E45" s="23" t="inlineStr">
+        <is>
+          <t>Tidewarden Coll (Ranged)</t>
+        </is>
+      </c>
+      <c r="F45" s="23" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="26" t="inlineStr">
+        <is>
+          <t>Perfectly Calm</t>
+        </is>
+      </c>
+      <c r="B46" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C46" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Water · Air</t>
+        </is>
+      </c>
+      <c r="E46" s="23" t="inlineStr">
+        <is>
+          <t>Nix (Ranged)</t>
+        </is>
+      </c>
+      <c r="F46" s="23" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="26" t="inlineStr">
+        <is>
+          <t>The Gaze Accuses</t>
+        </is>
+      </c>
+      <c r="B47" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C47" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Light · Fire</t>
+        </is>
+      </c>
+      <c r="E47" s="23" t="inlineStr">
+        <is>
+          <t>Seraphel (Striker)</t>
+        </is>
+      </c>
+      <c r="F47" s="23" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="26" t="inlineStr">
+        <is>
+          <t>Three Beams, No Shadow</t>
+        </is>
+      </c>
+      <c r="B48" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C48" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Light · Air</t>
+        </is>
+      </c>
+      <c r="E48" s="23" t="inlineStr">
+        <is>
+          <t>Lucen (Buffer)</t>
+        </is>
+      </c>
+      <c r="F48" s="23" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="26" t="inlineStr">
+        <is>
+          <t>The Lantern Holds</t>
+        </is>
+      </c>
+      <c r="B49" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C49" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Light · Water</t>
+        </is>
+      </c>
+      <c r="E49" s="23" t="inlineStr">
+        <is>
+          <t>Auriel Dawnkeep (Tank)</t>
+        </is>
+      </c>
+      <c r="F49" s="23" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="26" t="inlineStr">
+        <is>
+          <t>A Kindness, Ending</t>
+        </is>
+      </c>
+      <c r="B50" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C50" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Dark · Water</t>
+        </is>
+      </c>
+      <c r="E50" s="23" t="inlineStr">
+        <is>
+          <t>Nyxara (Striker)</t>
+        </is>
+      </c>
+      <c r="F50" s="23" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="26" t="inlineStr">
+        <is>
+          <t>Unwrite the Line</t>
+        </is>
+      </c>
+      <c r="B51" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C51" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Dark · Fire</t>
+        </is>
+      </c>
+      <c r="E51" s="23" t="inlineStr">
+        <is>
+          <t>Umbriel (Buffer)</t>
+        </is>
+      </c>
+      <c r="F51" s="23" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="26" t="inlineStr">
+        <is>
+          <t>I Know Your Hour</t>
+        </is>
+      </c>
+      <c r="B52" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C52" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Dark · Earth</t>
+        </is>
+      </c>
+      <c r="E52" s="23" t="inlineStr">
+        <is>
+          <t>Corvane (Tank)</t>
+        </is>
+      </c>
+      <c r="F52" s="23" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="26" t="inlineStr">
+        <is>
+          <t>Never Twice</t>
+        </is>
+      </c>
+      <c r="B53" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C53" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Slash · Light</t>
+        </is>
+      </c>
+      <c r="E53" s="23" t="inlineStr">
+        <is>
+          <t>Kaellis (Striker)</t>
+        </is>
+      </c>
+      <c r="F53" s="23" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="26" t="inlineStr">
+        <is>
+          <t>Two Rivers Meeting</t>
+        </is>
+      </c>
+      <c r="B54" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C54" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Slash · Water</t>
+        </is>
+      </c>
+      <c r="E54" s="23" t="inlineStr">
+        <is>
+          <t>Reyna Two-Rivers (Striker)</t>
+        </is>
+      </c>
+      <c r="F54" s="23" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="26" t="inlineStr">
+        <is>
+          <t>Clear the Room</t>
+        </is>
+      </c>
+      <c r="B55" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C55" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Slash · Dark</t>
+        </is>
+      </c>
+      <c r="E55" s="23" t="inlineStr">
+        <is>
+          <t>Grieve (Tank)</t>
+        </is>
+      </c>
+      <c r="F55" s="23" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="26" t="inlineStr">
+        <is>
+          <t>The One Gap</t>
+        </is>
+      </c>
+      <c r="B56" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C56" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Pierce · Air</t>
+        </is>
+      </c>
+      <c r="E56" s="23" t="inlineStr">
+        <is>
+          <t>Vantric (Striker)</t>
+        </is>
+      </c>
+      <c r="F56" s="23" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="26" t="inlineStr">
+        <is>
+          <t>Already Behind You</t>
+        </is>
+      </c>
+      <c r="B57" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C57" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Pierce · Dark</t>
+        </is>
+      </c>
+      <c r="E57" s="23" t="inlineStr">
+        <is>
+          <t>Silka Pinquick (Striker)</t>
+        </is>
+      </c>
+      <c r="F57" s="23" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="26" t="inlineStr">
+        <is>
+          <t>Before You Decide</t>
+        </is>
+      </c>
+      <c r="B58" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C58" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Pierce · Light</t>
+        </is>
+      </c>
+      <c r="E58" s="23" t="inlineStr">
+        <is>
+          <t>Lord Aiguille (Tank)</t>
+        </is>
+      </c>
+      <c r="F58" s="23" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="26" t="inlineStr">
+        <is>
+          <t>All At Once</t>
+        </is>
+      </c>
+      <c r="B59" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C59" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Crush · Light</t>
+        </is>
+      </c>
+      <c r="E59" s="23" t="inlineStr">
+        <is>
+          <t>Boldrek (Striker)</t>
+        </is>
+      </c>
+      <c r="F59" s="23" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="26" t="inlineStr">
+        <is>
+          <t>End of Argument</t>
+        </is>
+      </c>
+      <c r="B60" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C60" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Crush · Dark</t>
+        </is>
+      </c>
+      <c r="E60" s="23" t="inlineStr">
+        <is>
+          <t>Hettamar Ironfall (Striker)</t>
+        </is>
+      </c>
+      <c r="F60" s="23" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="26" t="inlineStr">
+        <is>
+          <t>Guards Break First</t>
+        </is>
+      </c>
+      <c r="B61" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C61" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Crush · Earth</t>
+        </is>
+      </c>
+      <c r="E61" s="23" t="inlineStr">
+        <is>
+          <t>Mauless (Tank)</t>
+        </is>
+      </c>
+      <c r="F61" s="23" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="26" t="inlineStr">
+        <is>
+          <t>Wrath of the Slow Stone</t>
+        </is>
+      </c>
+      <c r="B62" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C62" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Earth · Fire</t>
+        </is>
+      </c>
+      <c r="E62" s="23" t="inlineStr">
+        <is>
+          <t>Bramwen (Striker)</t>
+        </is>
+      </c>
+      <c r="F62" s="23" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="26" t="inlineStr">
+        <is>
+          <t>The God-Bone Wakes</t>
+        </is>
+      </c>
+      <c r="B63" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C63" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Earth · Dark</t>
+        </is>
+      </c>
+      <c r="E63" s="23" t="inlineStr">
+        <is>
+          <t>Ossic (Tank)</t>
+        </is>
+      </c>
+      <c r="F63" s="23" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="26" t="inlineStr">
+        <is>
+          <t>The Green Crown Descends</t>
+        </is>
+      </c>
+      <c r="B64" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C64" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Earth · Light</t>
+        </is>
+      </c>
+      <c r="E64" s="23" t="inlineStr">
+        <is>
+          <t>Terragosa (Tank)</t>
+        </is>
+      </c>
+      <c r="F64" s="23" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="26" t="inlineStr">
+        <is>
+          <t>The Thin Blade Falls</t>
+        </is>
+      </c>
+      <c r="B65" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C65" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Air · Light</t>
+        </is>
+      </c>
+      <c r="E65" s="23" t="inlineStr">
+        <is>
+          <t>Zephyrine (Striker)</t>
+        </is>
+      </c>
+      <c r="F65" s="23" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="26" t="inlineStr">
+        <is>
+          <t>Whisper from the High Reach</t>
+        </is>
+      </c>
+      <c r="B66" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C66" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Air · Water</t>
+        </is>
+      </c>
+      <c r="E66" s="23" t="inlineStr">
+        <is>
+          <t>Cirrolan (Buffer)</t>
+        </is>
+      </c>
+      <c r="F66" s="23" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="26" t="inlineStr">
+        <is>
+          <t>Nothing to Catch You</t>
+        </is>
+      </c>
+      <c r="B67" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C67" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Air · Dark</t>
+        </is>
+      </c>
+      <c r="E67" s="23" t="inlineStr">
+        <is>
+          <t>Vael (Ranged)</t>
+        </is>
+      </c>
+      <c r="F67" s="23" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="26" t="inlineStr">
+        <is>
+          <t>First Spark, Last Laugh</t>
+        </is>
+      </c>
+      <c r="B68" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C68" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Fire · Air</t>
+        </is>
+      </c>
+      <c r="E68" s="23" t="inlineStr">
+        <is>
+          <t>Ember Saelith (Striker)</t>
+        </is>
+      </c>
+      <c r="F68" s="23" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="26" t="inlineStr">
+        <is>
+          <t>Glad Ruin</t>
+        </is>
+      </c>
+      <c r="B69" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C69" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Fire · Light</t>
+        </is>
+      </c>
+      <c r="E69" s="23" t="inlineStr">
+        <is>
+          <t>Pyrrhic (Ranged)</t>
+        </is>
+      </c>
+      <c r="F69" s="23" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="26" t="inlineStr">
+        <is>
+          <t>The Long Burn</t>
+        </is>
+      </c>
+      <c r="B70" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C70" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Fire · Earth</t>
+        </is>
+      </c>
+      <c r="E70" s="23" t="inlineStr">
+        <is>
+          <t>Cindara (Ranged)</t>
+        </is>
+      </c>
+      <c r="F70" s="23" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="26" t="inlineStr">
+        <is>
+          <t>Drown in What You Did</t>
+        </is>
+      </c>
+      <c r="B71" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C71" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Water · Dark</t>
+        </is>
+      </c>
+      <c r="E71" s="23" t="inlineStr">
+        <is>
+          <t>Marisel (Striker)</t>
+        </is>
+      </c>
+      <c r="F71" s="23" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="26" t="inlineStr">
+        <is>
+          <t>The Bulwark Holds</t>
+        </is>
+      </c>
+      <c r="B72" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C72" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Water · Earth</t>
+        </is>
+      </c>
+      <c r="E72" s="23" t="inlineStr">
+        <is>
+          <t>Tidewarden Coll (Ranged)</t>
+        </is>
+      </c>
+      <c r="F72" s="23" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="26" t="inlineStr">
+        <is>
+          <t>The Still Pool Closes</t>
+        </is>
+      </c>
+      <c r="B73" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C73" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Water · Air</t>
+        </is>
+      </c>
+      <c r="E73" s="23" t="inlineStr">
+        <is>
+          <t>Nix (Ranged)</t>
+        </is>
+      </c>
+      <c r="F73" s="23" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="26" t="inlineStr">
+        <is>
+          <t>Sentence Passed</t>
+        </is>
+      </c>
+      <c r="B74" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C74" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Light · Fire</t>
+        </is>
+      </c>
+      <c r="E74" s="23" t="inlineStr">
+        <is>
+          <t>Seraphel (Striker)</t>
+        </is>
+      </c>
+      <c r="F74" s="23" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="26" t="inlineStr">
+        <is>
+          <t>The Unhidden Hour</t>
+        </is>
+      </c>
+      <c r="B75" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C75" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Light · Air</t>
+        </is>
+      </c>
+      <c r="E75" s="23" t="inlineStr">
+        <is>
+          <t>Lucen (Buffer)</t>
+        </is>
+      </c>
+      <c r="F75" s="23" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="26" t="inlineStr">
+        <is>
+          <t>Last Light on the Wall</t>
+        </is>
+      </c>
+      <c r="B76" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C76" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Light · Water</t>
+        </is>
+      </c>
+      <c r="E76" s="23" t="inlineStr">
+        <is>
+          <t>Auriel Dawnkeep (Tank)</t>
+        </is>
+      </c>
+      <c r="F76" s="23" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="26" t="inlineStr">
+        <is>
+          <t>Mercy at the End</t>
+        </is>
+      </c>
+      <c r="B77" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C77" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Dark · Water</t>
+        </is>
+      </c>
+      <c r="E77" s="23" t="inlineStr">
+        <is>
+          <t>Nyxara (Striker)</t>
+        </is>
+      </c>
+      <c r="F77" s="23" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="26" t="inlineStr">
+        <is>
+          <t>The Undoing</t>
+        </is>
+      </c>
+      <c r="B78" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C78" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Dark · Fire</t>
+        </is>
+      </c>
+      <c r="E78" s="23" t="inlineStr">
+        <is>
+          <t>Umbriel (Buffer)</t>
+        </is>
+      </c>
+      <c r="F78" s="23" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="26" t="inlineStr">
+        <is>
+          <t>Shepherd of Endings</t>
+        </is>
+      </c>
+      <c r="B79" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C79" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Dark · Earth</t>
+        </is>
+      </c>
+      <c r="E79" s="23" t="inlineStr">
+        <is>
+          <t>Corvane (Tank)</t>
+        </is>
+      </c>
+      <c r="F79" s="23" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="26" t="inlineStr">
+        <is>
+          <t>Immaculate</t>
+        </is>
+      </c>
+      <c r="B80" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C80" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Slash · Light</t>
+        </is>
+      </c>
+      <c r="E80" s="23" t="inlineStr">
+        <is>
+          <t>Kaellis (Striker)</t>
+        </is>
+      </c>
+      <c r="F80" s="23" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="26" t="inlineStr">
+        <is>
+          <t>The Current Takes All</t>
+        </is>
+      </c>
+      <c r="B81" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C81" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Slash · Water</t>
+        </is>
+      </c>
+      <c r="E81" s="23" t="inlineStr">
+        <is>
+          <t>Reyna Two-Rivers (Striker)</t>
+        </is>
+      </c>
+      <c r="F81" s="23" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="26" t="inlineStr">
+        <is>
+          <t>The Wide Reaping</t>
+        </is>
+      </c>
+      <c r="B82" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C82" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Slash · Dark</t>
+        </is>
+      </c>
+      <c r="E82" s="23" t="inlineStr">
+        <is>
+          <t>Grieve (Tank)</t>
+        </is>
+      </c>
+      <c r="F82" s="23" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="26" t="inlineStr">
+        <is>
+          <t>The Spear Finds It</t>
+        </is>
+      </c>
+      <c r="B83" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C83" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Pierce · Air</t>
+        </is>
+      </c>
+      <c r="E83" s="23" t="inlineStr">
+        <is>
+          <t>Vantric (Striker)</t>
+        </is>
+      </c>
+      <c r="F83" s="23" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="26" t="inlineStr">
+        <is>
+          <t>Quicker Than Told</t>
+        </is>
+      </c>
+      <c r="B84" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C84" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Pierce · Dark</t>
+        </is>
+      </c>
+      <c r="E84" s="23" t="inlineStr">
+        <is>
+          <t>Silka Pinquick (Striker)</t>
+        </is>
+      </c>
+      <c r="F84" s="23" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="26" t="inlineStr">
+        <is>
+          <t>The Long Point</t>
+        </is>
+      </c>
+      <c r="B85" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C85" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Pierce · Light</t>
+        </is>
+      </c>
+      <c r="E85" s="23" t="inlineStr">
+        <is>
+          <t>Lord Aiguille (Tank)</t>
+        </is>
+      </c>
+      <c r="F85" s="23" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="26" t="inlineStr">
+        <is>
+          <t>Avalanche</t>
+        </is>
+      </c>
+      <c r="B86" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C86" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Crush · Light</t>
+        </is>
+      </c>
+      <c r="E86" s="23" t="inlineStr">
+        <is>
+          <t>Boldrek (Striker)</t>
+        </is>
+      </c>
+      <c r="F86" s="23" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="26" t="inlineStr">
+        <is>
+          <t>Ironfall</t>
+        </is>
+      </c>
+      <c r="B87" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C87" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Crush · Dark</t>
+        </is>
+      </c>
+      <c r="E87" s="23" t="inlineStr">
+        <is>
+          <t>Hettamar Ironfall (Striker)</t>
+        </is>
+      </c>
+      <c r="F87" s="23" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="26" t="inlineStr">
+        <is>
+          <t>The Undenied</t>
+        </is>
+      </c>
+      <c r="B88" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C88" s="22" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Crush · Earth</t>
+        </is>
+      </c>
+      <c r="E88" s="23" t="inlineStr">
+        <is>
+          <t>Mauless (Tank)</t>
+        </is>
+      </c>
+      <c r="F88" s="23" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F88"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>